<commit_message>
Atualiza├º├úo autom├ítica 2025-10-16 10:14
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="289" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E42DE2A-A550-4A36-9234-25E01B1F72F5}"/>
+  <xr:revisionPtr revIDLastSave="303" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F6F3F9AB-7DA2-41FA-886D-5DE20A353326}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1757" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1763" uniqueCount="113">
   <si>
     <t>Custo</t>
   </si>
@@ -14196,25 +14196,49 @@
       </c>
     </row>
     <row r="878" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B878" s="11"/>
+      <c r="B878" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C878" s="5"/>
-      <c r="D878" s="3"/>
-      <c r="E878" s="19"/>
-      <c r="F878" s="7"/>
+      <c r="D878" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E878" s="19">
+        <v>802.61</v>
+      </c>
+      <c r="F878" s="7">
+        <v>45931</v>
+      </c>
     </row>
     <row r="879" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B879" s="11"/>
+      <c r="B879" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C879" s="5"/>
-      <c r="D879" s="3"/>
-      <c r="E879" s="19"/>
-      <c r="F879" s="7"/>
+      <c r="D879" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E879" s="19">
+        <v>229.89</v>
+      </c>
+      <c r="F879" s="7">
+        <v>45931</v>
+      </c>
     </row>
     <row r="880" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B880" s="11"/>
+      <c r="B880" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C880" s="5"/>
-      <c r="D880" s="3"/>
-      <c r="E880" s="19"/>
-      <c r="F880" s="7"/>
+      <c r="D880" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E880" s="19">
+        <v>1558.88</v>
+      </c>
+      <c r="F880" s="7">
+        <v>45931</v>
+      </c>
     </row>
     <row r="881" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B881" s="11"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-10-27 17:09
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="380" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8D476208-1DAD-4259-924C-853928F04D33}"/>
+  <xr:revisionPtr revIDLastSave="384" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8440537-1EF3-4AAF-9038-977A2F4FF466}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1797" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1799" uniqueCount="115">
   <si>
     <t>Custo</t>
   </si>
@@ -14503,11 +14503,19 @@
       </c>
     </row>
     <row r="898" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B898" s="11"/>
+      <c r="B898" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C898" s="5"/>
-      <c r="D898" s="3"/>
-      <c r="E898" s="19"/>
-      <c r="F898" s="7"/>
+      <c r="D898" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E898" s="19">
+        <v>310</v>
+      </c>
+      <c r="F898" s="7">
+        <v>45931</v>
+      </c>
     </row>
     <row r="899" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B899" s="11"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-24  9:27
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="551" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8A5ED4E6-0AD1-4423-8FFE-BCD989E2C857}"/>
+  <xr:revisionPtr revIDLastSave="700" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E98BBA67-7AE7-4922-95D3-D12C181226CF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1963" uniqueCount="120">
   <si>
     <t>Custo</t>
   </si>
@@ -393,6 +393,12 @@
   </si>
   <si>
     <t>LINHA CARROCERIAS</t>
+  </si>
+  <si>
+    <t>PCD7I11</t>
+  </si>
+  <si>
+    <t>SIDER DIVI</t>
   </si>
 </sst>
 </file>
@@ -15152,291 +15158,619 @@
       </c>
     </row>
     <row r="940" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B940" s="11"/>
+      <c r="B940" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C940" s="5"/>
-      <c r="D940" s="3"/>
-      <c r="E940" s="19"/>
-      <c r="F940" s="7"/>
+      <c r="D940" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E940" s="19">
+        <v>220</v>
+      </c>
+      <c r="F940" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="941" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B941" s="11"/>
+      <c r="B941" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C941" s="5"/>
-      <c r="D941" s="3"/>
-      <c r="E941" s="19"/>
-      <c r="F941" s="7"/>
+      <c r="D941" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E941" s="19">
+        <v>48</v>
+      </c>
+      <c r="F941" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="942" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B942" s="11"/>
+      <c r="B942" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C942" s="5"/>
-      <c r="D942" s="3"/>
-      <c r="E942" s="19"/>
-      <c r="F942" s="7"/>
+      <c r="D942" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E942" s="19">
+        <v>501.2</v>
+      </c>
+      <c r="F942" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="943" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B943" s="11"/>
+      <c r="B943" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C943" s="5"/>
-      <c r="D943" s="3"/>
-      <c r="E943" s="19"/>
-      <c r="F943" s="7"/>
+      <c r="D943" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E943" s="19">
+        <v>15</v>
+      </c>
+      <c r="F943" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="944" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B944" s="11"/>
+      <c r="B944" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C944" s="5"/>
-      <c r="D944" s="3"/>
-      <c r="E944" s="19"/>
-      <c r="F944" s="7"/>
+      <c r="D944" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E944" s="19">
+        <v>375</v>
+      </c>
+      <c r="F944" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="945" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B945" s="11"/>
+      <c r="B945" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C945" s="5"/>
-      <c r="D945" s="3"/>
-      <c r="E945" s="19"/>
-      <c r="F945" s="7"/>
+      <c r="D945" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="E945" s="19">
+        <v>270</v>
+      </c>
+      <c r="F945" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="946" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B946" s="11"/>
+      <c r="B946" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C946" s="5"/>
-      <c r="D946" s="3"/>
-      <c r="E946" s="19"/>
-      <c r="F946" s="7"/>
+      <c r="D946" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E946" s="19">
+        <v>130</v>
+      </c>
+      <c r="F946" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="947" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B947" s="11"/>
+      <c r="B947" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C947" s="5"/>
-      <c r="D947" s="3"/>
-      <c r="E947" s="19"/>
-      <c r="F947" s="7"/>
+      <c r="D947" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="E947" s="19">
+        <v>390.01</v>
+      </c>
+      <c r="F947" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="948" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B948" s="11"/>
+      <c r="B948" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C948" s="5"/>
-      <c r="D948" s="3"/>
-      <c r="E948" s="19"/>
-      <c r="F948" s="7"/>
+      <c r="D948" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="E948" s="19">
+        <v>3300</v>
+      </c>
+      <c r="F948" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="949" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B949" s="11"/>
+      <c r="B949" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C949" s="5"/>
-      <c r="D949" s="3"/>
-      <c r="E949" s="19"/>
-      <c r="F949" s="7"/>
+      <c r="D949" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E949" s="19">
+        <v>280</v>
+      </c>
+      <c r="F949" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="950" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B950" s="11"/>
+      <c r="B950" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C950" s="5"/>
-      <c r="D950" s="3"/>
-      <c r="E950" s="19"/>
-      <c r="F950" s="7"/>
+      <c r="D950" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E950" s="19">
+        <v>280</v>
+      </c>
+      <c r="F950" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="951" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B951" s="11"/>
+      <c r="B951" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C951" s="5"/>
-      <c r="D951" s="3"/>
-      <c r="E951" s="19"/>
-      <c r="F951" s="7"/>
+      <c r="D951" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E951" s="19">
+        <v>775</v>
+      </c>
+      <c r="F951" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="952" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B952" s="11"/>
+      <c r="B952" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C952" s="5"/>
-      <c r="D952" s="3"/>
-      <c r="E952" s="19"/>
-      <c r="F952" s="7"/>
+      <c r="D952" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E952" s="19">
+        <v>80</v>
+      </c>
+      <c r="F952" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="953" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B953" s="11"/>
+      <c r="B953" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="C953" s="5"/>
-      <c r="D953" s="3"/>
-      <c r="E953" s="19"/>
-      <c r="F953" s="7"/>
+      <c r="D953" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E953" s="19">
+        <v>250</v>
+      </c>
+      <c r="F953" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="954" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B954" s="11"/>
+      <c r="B954" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C954" s="5"/>
-      <c r="D954" s="3"/>
-      <c r="E954" s="19"/>
-      <c r="F954" s="7"/>
+      <c r="D954" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E954" s="19">
+        <v>200</v>
+      </c>
+      <c r="F954" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="955" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B955" s="11"/>
+      <c r="B955" s="11" t="s">
+        <v>118</v>
+      </c>
       <c r="C955" s="5"/>
-      <c r="D955" s="3"/>
-      <c r="E955" s="19"/>
-      <c r="F955" s="7"/>
+      <c r="D955" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E955" s="19">
+        <v>609.75</v>
+      </c>
+      <c r="F955" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="956" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B956" s="11"/>
+      <c r="B956" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C956" s="5"/>
-      <c r="D956" s="3"/>
-      <c r="E956" s="19"/>
-      <c r="F956" s="7"/>
+      <c r="D956" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E956" s="19">
+        <v>1062</v>
+      </c>
+      <c r="F956" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="957" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B957" s="11"/>
+      <c r="B957" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C957" s="5"/>
-      <c r="D957" s="3"/>
-      <c r="E957" s="19"/>
-      <c r="F957" s="7"/>
+      <c r="D957" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="E957" s="19">
+        <v>2347.44</v>
+      </c>
+      <c r="F957" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="958" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B958" s="11"/>
+      <c r="B958" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C958" s="5"/>
-      <c r="D958" s="3"/>
-      <c r="E958" s="19"/>
-      <c r="F958" s="7"/>
+      <c r="D958" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E958" s="19">
+        <v>44</v>
+      </c>
+      <c r="F958" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="959" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B959" s="11"/>
+      <c r="B959" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="C959" s="5"/>
-      <c r="D959" s="3"/>
-      <c r="E959" s="19"/>
-      <c r="F959" s="7"/>
+      <c r="D959" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E959" s="19">
+        <v>200</v>
+      </c>
+      <c r="F959" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="960" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B960" s="11"/>
+      <c r="B960" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C960" s="5"/>
-      <c r="D960" s="3"/>
-      <c r="E960" s="19"/>
-      <c r="F960" s="7"/>
+      <c r="D960" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="E960" s="19">
+        <v>20</v>
+      </c>
+      <c r="F960" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="961" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B961" s="11"/>
+      <c r="B961" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C961" s="5"/>
-      <c r="D961" s="3"/>
-      <c r="E961" s="19"/>
-      <c r="F961" s="7"/>
+      <c r="D961" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E961" s="19">
+        <v>780</v>
+      </c>
+      <c r="F961" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="962" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B962" s="11"/>
+      <c r="B962" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C962" s="5"/>
-      <c r="D962" s="3"/>
-      <c r="E962" s="19"/>
-      <c r="F962" s="7"/>
+      <c r="D962" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E962" s="19">
+        <v>370</v>
+      </c>
+      <c r="F962" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="963" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B963" s="11"/>
+      <c r="B963" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C963" s="5"/>
-      <c r="D963" s="3"/>
-      <c r="E963" s="19"/>
-      <c r="F963" s="7"/>
+      <c r="D963" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E963" s="19">
+        <v>540</v>
+      </c>
+      <c r="F963" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="964" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B964" s="11"/>
+      <c r="B964" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C964" s="5"/>
-      <c r="D964" s="3"/>
-      <c r="E964" s="19"/>
-      <c r="F964" s="7"/>
+      <c r="D964" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E964" s="19">
+        <v>318</v>
+      </c>
+      <c r="F964" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="965" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B965" s="11"/>
+      <c r="B965" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C965" s="5"/>
-      <c r="D965" s="3"/>
-      <c r="E965" s="19"/>
-      <c r="F965" s="7"/>
+      <c r="D965" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E965" s="19">
+        <v>590</v>
+      </c>
+      <c r="F965" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="966" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B966" s="11"/>
+      <c r="B966" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C966" s="5"/>
-      <c r="D966" s="3"/>
-      <c r="E966" s="19"/>
-      <c r="F966" s="7"/>
+      <c r="D966" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E966" s="19">
+        <v>120</v>
+      </c>
+      <c r="F966" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="967" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B967" s="11"/>
+      <c r="B967" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C967" s="5"/>
-      <c r="D967" s="3"/>
-      <c r="E967" s="19"/>
-      <c r="F967" s="7"/>
+      <c r="D967" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E967" s="19">
+        <v>3369.52</v>
+      </c>
+      <c r="F967" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="968" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B968" s="11"/>
+      <c r="B968" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C968" s="5"/>
-      <c r="D968" s="3"/>
-      <c r="E968" s="19"/>
-      <c r="F968" s="7"/>
+      <c r="D968" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E968" s="19">
+        <v>80</v>
+      </c>
+      <c r="F968" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="969" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B969" s="11"/>
+      <c r="B969" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C969" s="5"/>
-      <c r="D969" s="3"/>
-      <c r="E969" s="19"/>
-      <c r="F969" s="7"/>
+      <c r="D969" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="E969" s="19">
+        <v>300</v>
+      </c>
+      <c r="F969" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="970" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B970" s="11"/>
+      <c r="B970" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C970" s="5"/>
-      <c r="D970" s="3"/>
-      <c r="E970" s="19"/>
-      <c r="F970" s="7"/>
+      <c r="D970" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E970" s="19">
+        <v>280</v>
+      </c>
+      <c r="F970" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="971" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B971" s="11"/>
+      <c r="B971" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C971" s="5"/>
-      <c r="D971" s="3"/>
-      <c r="E971" s="19"/>
-      <c r="F971" s="7"/>
+      <c r="D971" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E971" s="19">
+        <v>100</v>
+      </c>
+      <c r="F971" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="972" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B972" s="11"/>
+      <c r="B972" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C972" s="5"/>
-      <c r="D972" s="3"/>
-      <c r="E972" s="19"/>
-      <c r="F972" s="7"/>
+      <c r="D972" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E972" s="19">
+        <v>902.1</v>
+      </c>
+      <c r="F972" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="973" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B973" s="11"/>
+      <c r="B973" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C973" s="5"/>
-      <c r="D973" s="3"/>
-      <c r="E973" s="19"/>
-      <c r="F973" s="7"/>
+      <c r="D973" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E973" s="19">
+        <v>605.6</v>
+      </c>
+      <c r="F973" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="974" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B974" s="11"/>
+      <c r="B974" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C974" s="5"/>
-      <c r="D974" s="3"/>
-      <c r="E974" s="19"/>
-      <c r="F974" s="7"/>
+      <c r="D974" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E974" s="19">
+        <v>735</v>
+      </c>
+      <c r="F974" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="975" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B975" s="11"/>
+      <c r="B975" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C975" s="5"/>
-      <c r="D975" s="3"/>
-      <c r="E975" s="19"/>
-      <c r="F975" s="7"/>
+      <c r="D975" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E975" s="19">
+        <v>200</v>
+      </c>
+      <c r="F975" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="976" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B976" s="11"/>
+      <c r="B976" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="C976" s="5"/>
-      <c r="D976" s="3"/>
-      <c r="E976" s="19"/>
-      <c r="F976" s="7"/>
+      <c r="D976" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E976" s="19">
+        <v>265</v>
+      </c>
+      <c r="F976" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="977" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B977" s="11"/>
+      <c r="B977" s="11" t="s">
+        <v>118</v>
+      </c>
       <c r="C977" s="5"/>
-      <c r="D977" s="3"/>
-      <c r="E977" s="19"/>
-      <c r="F977" s="7"/>
+      <c r="D977" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E977" s="19">
+        <v>1040</v>
+      </c>
+      <c r="F977" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="978" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B978" s="11"/>
+      <c r="B978" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C978" s="5"/>
-      <c r="D978" s="3"/>
-      <c r="E978" s="19"/>
-      <c r="F978" s="7"/>
+      <c r="D978" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E978" s="19">
+        <v>445.2</v>
+      </c>
+      <c r="F978" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="979" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B979" s="11"/>
+      <c r="B979" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C979" s="5"/>
-      <c r="D979" s="3"/>
-      <c r="E979" s="19"/>
-      <c r="F979" s="7"/>
+      <c r="D979" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E979" s="19">
+        <v>90</v>
+      </c>
+      <c r="F979" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="980" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B980" s="11"/>
+      <c r="B980" s="11" t="s">
+        <v>101</v>
+      </c>
       <c r="C980" s="5"/>
-      <c r="D980" s="3"/>
-      <c r="E980" s="19"/>
-      <c r="F980" s="7"/>
+      <c r="D980" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E980" s="19">
+        <v>395</v>
+      </c>
+      <c r="F980" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="981" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B981" s="11"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-27 15:17
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="746" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C868B7CC-E4B5-4277-93B5-EA9F3859AB5F}"/>
+  <xr:revisionPtr revIDLastSave="750" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21EEB557-9956-41EB-8D78-DA435AF30C8D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1989" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1991" uniqueCount="124">
   <si>
     <t>Custo</t>
   </si>
@@ -15980,11 +15980,19 @@
       </c>
     </row>
     <row r="994" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B994" s="11"/>
+      <c r="B994" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C994" s="5"/>
-      <c r="D994" s="3"/>
-      <c r="E994" s="19"/>
-      <c r="F994" s="7"/>
+      <c r="D994" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="E994" s="19">
+        <v>1980</v>
+      </c>
+      <c r="F994" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="995" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B995" s="11"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-27 15:23
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/jhonatan_veiga_jrferragens_com/Documents/01/HTML/DASHBOARD/DASHBOARD/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="750" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21EEB557-9956-41EB-8D78-DA435AF30C8D}"/>
+  <xr:revisionPtr revIDLastSave="754" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E62DF2A2-6EEB-4FEC-8CD4-7E0BE1F40E22}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1991" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1993" uniqueCount="124">
   <si>
     <t>Custo</t>
   </si>
@@ -15995,11 +15995,19 @@
       </c>
     </row>
     <row r="995" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B995" s="11"/>
+      <c r="B995" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C995" s="5"/>
-      <c r="D995" s="3"/>
-      <c r="E995" s="19"/>
-      <c r="F995" s="7"/>
+      <c r="D995" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E995" s="19">
+        <v>325</v>
+      </c>
+      <c r="F995" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="996" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B996" s="11"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-11-27 15:41
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="754" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E62DF2A2-6EEB-4FEC-8CD4-7E0BE1F40E22}"/>
+  <xr:revisionPtr revIDLastSave="758" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77E6D82B-5751-485E-B0CF-A0FE39103534}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1993" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="124">
   <si>
     <t>Custo</t>
   </si>
@@ -16010,11 +16010,19 @@
       </c>
     </row>
     <row r="996" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B996" s="11"/>
+      <c r="B996" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C996" s="5"/>
-      <c r="D996" s="3"/>
-      <c r="E996" s="19"/>
-      <c r="F996" s="7"/>
+      <c r="D996" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E996" s="19">
+        <v>136.35</v>
+      </c>
+      <c r="F996" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="997" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B997" s="11"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-12-01 17:25
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="758" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77E6D82B-5751-485E-B0CF-A0FE39103534}"/>
+  <xr:revisionPtr revIDLastSave="769" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A398A076-F07D-4EB3-98F6-F9231AD2B90B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1995" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1999" uniqueCount="124">
   <si>
     <t>Custo</t>
   </si>
@@ -420,7 +420,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,6 +451,14 @@
     </font>
     <font>
       <u val="singleAccounting"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
@@ -646,7 +654,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -752,6 +760,7 @@
     <xf numFmtId="44" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
@@ -15964,7 +15973,7 @@
         <v>45962</v>
       </c>
     </row>
-    <row r="993" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="993" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B993" s="11" t="s">
         <v>28</v>
       </c>
@@ -15979,7 +15988,7 @@
         <v>45962</v>
       </c>
     </row>
-    <row r="994" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="994" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B994" s="11" t="s">
         <v>28</v>
       </c>
@@ -15994,7 +16003,7 @@
         <v>45962</v>
       </c>
     </row>
-    <row r="995" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="995" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B995" s="11" t="s">
         <v>22</v>
       </c>
@@ -16009,7 +16018,7 @@
         <v>45962</v>
       </c>
     </row>
-    <row r="996" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="996" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B996" s="11" t="s">
         <v>11</v>
       </c>
@@ -16024,84 +16033,101 @@
         <v>45962</v>
       </c>
     </row>
-    <row r="997" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B997" s="11"/>
+    <row r="997" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B997" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C997" s="5"/>
-      <c r="D997" s="3"/>
-      <c r="E997" s="19"/>
-      <c r="F997" s="7"/>
-    </row>
-    <row r="998" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B998" s="11"/>
+      <c r="D997" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="E997" s="19">
+        <v>2176.25</v>
+      </c>
+      <c r="F997" s="7">
+        <v>45962</v>
+      </c>
+      <c r="G997" s="41"/>
+    </row>
+    <row r="998" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B998" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C998" s="5"/>
-      <c r="D998" s="3"/>
-      <c r="E998" s="19"/>
-      <c r="F998" s="7"/>
-    </row>
-    <row r="999" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="D998" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="E998" s="19">
+        <v>560</v>
+      </c>
+      <c r="F998" s="7">
+        <v>45962</v>
+      </c>
+    </row>
+    <row r="999" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B999" s="11"/>
       <c r="C999" s="5"/>
       <c r="D999" s="3"/>
       <c r="E999" s="19"/>
       <c r="F999" s="7"/>
     </row>
-    <row r="1000" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1000" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1000" s="11"/>
       <c r="C1000" s="5"/>
       <c r="D1000" s="3"/>
       <c r="E1000" s="19"/>
       <c r="F1000" s="7"/>
     </row>
-    <row r="1001" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1001" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1001" s="11"/>
       <c r="C1001" s="5"/>
       <c r="D1001" s="3"/>
       <c r="E1001" s="19"/>
       <c r="F1001" s="7"/>
     </row>
-    <row r="1002" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1002" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1002" s="11"/>
       <c r="C1002" s="5"/>
       <c r="D1002" s="3"/>
       <c r="E1002" s="19"/>
       <c r="F1002" s="7"/>
     </row>
-    <row r="1003" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1003" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1003" s="11"/>
       <c r="C1003" s="5"/>
       <c r="D1003" s="3"/>
       <c r="E1003" s="19"/>
       <c r="F1003" s="7"/>
     </row>
-    <row r="1004" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1004" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1004" s="11"/>
       <c r="C1004" s="5"/>
       <c r="D1004" s="3"/>
       <c r="E1004" s="19"/>
       <c r="F1004" s="7"/>
     </row>
-    <row r="1005" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1005" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1005" s="11"/>
       <c r="C1005" s="5"/>
       <c r="D1005" s="3"/>
       <c r="E1005" s="19"/>
       <c r="F1005" s="7"/>
     </row>
-    <row r="1006" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1006" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1006" s="11"/>
       <c r="C1006" s="5"/>
       <c r="D1006" s="3"/>
       <c r="E1006" s="19"/>
       <c r="F1006" s="7"/>
     </row>
-    <row r="1007" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1007" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1007" s="11"/>
       <c r="C1007" s="5"/>
       <c r="D1007" s="3"/>
       <c r="E1007" s="19"/>
       <c r="F1007" s="7"/>
     </row>
-    <row r="1008" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="1008" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1008" s="11"/>
       <c r="C1008" s="5"/>
       <c r="D1008" s="3"/>

</xml_diff>

<commit_message>
Atualiza├º├úo autom├ítica 2025-12-03 15:43
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="769" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A398A076-F07D-4EB3-98F6-F9231AD2B90B}"/>
+  <xr:revisionPtr revIDLastSave="789" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{833B8943-5922-4ECE-B462-FCD736867601}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1999" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2007" uniqueCount="125">
   <si>
     <t>Custo</t>
   </si>
@@ -411,6 +411,9 @@
   </si>
   <si>
     <t xml:space="preserve">MS PNEUS </t>
+  </si>
+  <si>
+    <t>AUTO PECAS BD</t>
   </si>
 </sst>
 </file>
@@ -16065,32 +16068,65 @@
       </c>
     </row>
     <row r="999" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B999" s="11"/>
+      <c r="B999" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C999" s="5"/>
-      <c r="D999" s="3"/>
-      <c r="E999" s="19"/>
-      <c r="F999" s="7"/>
+      <c r="D999" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E999" s="19">
+        <v>1100</v>
+      </c>
+      <c r="F999" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="1000" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B1000" s="11"/>
+      <c r="B1000" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C1000" s="5"/>
-      <c r="D1000" s="3"/>
-      <c r="E1000" s="19"/>
-      <c r="F1000" s="7"/>
+      <c r="D1000" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1000" s="19">
+        <v>80</v>
+      </c>
+      <c r="F1000" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="1001" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B1001" s="11"/>
+      <c r="B1001" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C1001" s="5"/>
-      <c r="D1001" s="3"/>
-      <c r="E1001" s="19"/>
-      <c r="F1001" s="7"/>
+      <c r="D1001" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1001" s="19">
+        <v>280</v>
+      </c>
+      <c r="F1001" s="7">
+        <v>45962</v>
+      </c>
+      <c r="G1001" s="7"/>
     </row>
     <row r="1002" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B1002" s="11"/>
+      <c r="B1002" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C1002" s="5"/>
-      <c r="D1002" s="3"/>
-      <c r="E1002" s="19"/>
-      <c r="F1002" s="7"/>
+      <c r="D1002" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E1002" s="19">
+        <v>445</v>
+      </c>
+      <c r="F1002" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="1003" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B1003" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-06 17:31
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1083" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3019CEF-2731-4AD7-8CA8-858DD9090BE9}"/>
+  <xr:revisionPtr revIDLastSave="1142" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBF11876-99EB-4989-8126-B8350C5DE72A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2139" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2165" uniqueCount="134">
   <si>
     <t>Custo</t>
   </si>
@@ -437,6 +437,12 @@
   </si>
   <si>
     <t>KPD8B86</t>
+  </si>
+  <si>
+    <t>SEM INFORMAÇÃO</t>
+  </si>
+  <si>
+    <t>AG PNEUS</t>
   </si>
 </sst>
 </file>
@@ -17087,95 +17093,199 @@
       </c>
     </row>
     <row r="1066" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1066" s="11"/>
+      <c r="B1066" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C1066" s="5"/>
-      <c r="D1066" s="3"/>
-      <c r="E1066" s="19"/>
-      <c r="F1066" s="7"/>
+      <c r="D1066" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1066" s="19">
+        <v>555</v>
+      </c>
+      <c r="F1066" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1067" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1067" s="11"/>
+      <c r="B1067" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C1067" s="5"/>
-      <c r="D1067" s="3"/>
-      <c r="E1067" s="19"/>
-      <c r="F1067" s="7"/>
+      <c r="D1067" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1067" s="19">
+        <v>2600</v>
+      </c>
+      <c r="F1067" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1068" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1068" s="11"/>
+      <c r="B1068" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C1068" s="5"/>
-      <c r="D1068" s="3"/>
-      <c r="E1068" s="19"/>
-      <c r="F1068" s="7"/>
+      <c r="D1068" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E1068" s="19">
+        <v>220</v>
+      </c>
+      <c r="F1068" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1069" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1069" s="11"/>
+      <c r="B1069" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C1069" s="5"/>
-      <c r="D1069" s="3"/>
-      <c r="E1069" s="19"/>
-      <c r="F1069" s="7"/>
+      <c r="D1069" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1069" s="19">
+        <v>80</v>
+      </c>
+      <c r="F1069" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1070" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1070" s="11"/>
+      <c r="B1070" s="11" t="s">
+        <v>132</v>
+      </c>
       <c r="C1070" s="5"/>
-      <c r="D1070" s="3"/>
-      <c r="E1070" s="19"/>
-      <c r="F1070" s="7"/>
+      <c r="D1070" s="3" t="s">
+        <v>50</v>
+      </c>
+      <c r="E1070" s="19">
+        <v>702</v>
+      </c>
+      <c r="F1070" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1071" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1071" s="11"/>
+      <c r="B1071" s="11" t="s">
+        <v>92</v>
+      </c>
       <c r="C1071" s="5"/>
-      <c r="D1071" s="3"/>
-      <c r="E1071" s="19"/>
-      <c r="F1071" s="7"/>
+      <c r="D1071" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1071" s="19">
+        <v>540</v>
+      </c>
+      <c r="F1071" s="7">
+        <v>45962</v>
+      </c>
     </row>
     <row r="1072" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1072" s="11"/>
+      <c r="B1072" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C1072" s="5"/>
-      <c r="D1072" s="3"/>
-      <c r="E1072" s="19"/>
-      <c r="F1072" s="7"/>
+      <c r="D1072" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1072" s="19">
+        <v>495</v>
+      </c>
+      <c r="F1072" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1073" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1073" s="11"/>
+      <c r="B1073" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C1073" s="5"/>
-      <c r="D1073" s="3"/>
-      <c r="E1073" s="19"/>
-      <c r="F1073" s="7"/>
+      <c r="D1073" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E1073" s="19">
+        <v>1700</v>
+      </c>
+      <c r="F1073" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1074" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1074" s="11"/>
+      <c r="B1074" s="11" t="s">
+        <v>92</v>
+      </c>
       <c r="C1074" s="5"/>
-      <c r="D1074" s="3"/>
-      <c r="E1074" s="19"/>
-      <c r="F1074" s="7"/>
+      <c r="D1074" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1074" s="19">
+        <v>833</v>
+      </c>
+      <c r="F1074" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1075" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1075" s="11"/>
+      <c r="B1075" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C1075" s="5"/>
-      <c r="D1075" s="3"/>
-      <c r="E1075" s="19"/>
-      <c r="F1075" s="7"/>
+      <c r="D1075" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1075" s="19">
+        <v>265</v>
+      </c>
+      <c r="F1075" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1076" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1076" s="11"/>
+      <c r="B1076" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C1076" s="5"/>
-      <c r="D1076" s="3"/>
-      <c r="E1076" s="19"/>
-      <c r="F1076" s="7"/>
+      <c r="D1076" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E1076" s="19">
+        <v>3187</v>
+      </c>
+      <c r="F1076" s="7">
+        <v>45931</v>
+      </c>
     </row>
     <row r="1077" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1077" s="11"/>
+      <c r="B1077" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="C1077" s="5"/>
-      <c r="D1077" s="3"/>
-      <c r="E1077" s="19"/>
-      <c r="F1077" s="7"/>
+      <c r="D1077" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1077" s="19">
+        <v>1036</v>
+      </c>
+      <c r="F1077" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1078" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1078" s="11"/>
+      <c r="B1078" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C1078" s="5"/>
-      <c r="D1078" s="3"/>
-      <c r="E1078" s="19"/>
-      <c r="F1078" s="7"/>
+      <c r="D1078" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="E1078" s="19">
+        <v>690</v>
+      </c>
+      <c r="F1078" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1079" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1079" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-13 08:56
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1315" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{ABFDA1F5-E1BB-4A85-BCA6-A4CFC0D8349D}"/>
+  <xr:revisionPtr revIDLastSave="1323" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A36B252-B537-492E-A120-20979C95B190}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2233" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2237" uniqueCount="139">
   <si>
     <t>Custo</t>
   </si>
@@ -40064,18 +40064,34 @@
       </c>
     </row>
     <row r="39" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B39" s="11"/>
+      <c r="B39" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C39" s="5"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="19"/>
-      <c r="F39" s="7"/>
+      <c r="D39" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E39" s="19">
+        <v>1266.2</v>
+      </c>
+      <c r="F39" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="40" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B40" s="11"/>
+      <c r="B40" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C40" s="5"/>
-      <c r="D40" s="3"/>
-      <c r="E40" s="19"/>
-      <c r="F40" s="7"/>
+      <c r="D40" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E40" s="19">
+        <v>400</v>
+      </c>
+      <c r="F40" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B41" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-13 10:49
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1323" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A36B252-B537-492E-A120-20979C95B190}"/>
+  <xr:revisionPtr revIDLastSave="1331" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A443FB8B-9ACA-44F0-8084-22C19AE4F901}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2237" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2241" uniqueCount="140">
   <si>
     <t>Custo</t>
   </si>
@@ -458,6 +458,9 @@
   </si>
   <si>
     <t>REFORMA PNEU</t>
+  </si>
+  <si>
+    <t>CENTER TRUCK</t>
   </si>
 </sst>
 </file>
@@ -40094,18 +40097,34 @@
       </c>
     </row>
     <row r="41" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B41" s="11"/>
+      <c r="B41" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C41" s="5"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="19"/>
-      <c r="F41" s="7"/>
+      <c r="D41" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E41" s="19">
+        <v>8350</v>
+      </c>
+      <c r="F41" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="42" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B42" s="11"/>
+      <c r="B42" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="C42" s="5"/>
-      <c r="D42" s="3"/>
-      <c r="E42" s="19"/>
-      <c r="F42" s="7"/>
+      <c r="D42" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E42" s="19">
+        <v>3500</v>
+      </c>
+      <c r="F42" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B43" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-13 11:06
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1331" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A443FB8B-9ACA-44F0-8084-22C19AE4F901}"/>
+  <xr:revisionPtr revIDLastSave="1335" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{557AD426-6476-4D02-8663-F55208043EA1}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
+    <workbookView xWindow="7560" yWindow="3555" windowWidth="18345" windowHeight="11295" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2241" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2243" uniqueCount="140">
   <si>
     <t>Custo</t>
   </si>
@@ -40127,11 +40127,19 @@
       </c>
     </row>
     <row r="43" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B43" s="11"/>
+      <c r="B43" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C43" s="5"/>
-      <c r="D43" s="3"/>
-      <c r="E43" s="19"/>
-      <c r="F43" s="7"/>
+      <c r="D43" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E43" s="19">
+        <v>798.3</v>
+      </c>
+      <c r="F43" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="44" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B44" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-01-27 16:49
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1496" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B331250A-A2B8-4DBD-9139-4C72F4A711B5}"/>
+  <xr:revisionPtr revIDLastSave="1524" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{541D4054-AF43-4099-8FA6-0B4EFEEDB118}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2315" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2329" uniqueCount="147">
   <si>
     <t>Custo</t>
   </si>
@@ -40710,53 +40710,109 @@
       </c>
     </row>
     <row r="79" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B79" s="11"/>
+      <c r="B79" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C79" s="5"/>
-      <c r="D79" s="3"/>
-      <c r="E79" s="43"/>
-      <c r="F79" s="7"/>
+      <c r="D79" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E79" s="43">
+        <v>300</v>
+      </c>
+      <c r="F79" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="80" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B80" s="11"/>
+      <c r="B80" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C80" s="5"/>
-      <c r="D80" s="3"/>
-      <c r="E80" s="43"/>
-      <c r="F80" s="7"/>
+      <c r="D80" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E80" s="43">
+        <v>37.6</v>
+      </c>
+      <c r="F80" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="81" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B81" s="11"/>
+      <c r="B81" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C81" s="5"/>
-      <c r="D81" s="3"/>
-      <c r="E81" s="43"/>
-      <c r="F81" s="7"/>
+      <c r="D81" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E81" s="43">
+        <v>760</v>
+      </c>
+      <c r="F81" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="82" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B82" s="11"/>
+      <c r="B82" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C82" s="5"/>
-      <c r="D82" s="3"/>
-      <c r="E82" s="43"/>
-      <c r="F82" s="7"/>
+      <c r="D82" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E82" s="43">
+        <v>100</v>
+      </c>
+      <c r="F82" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="83" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B83" s="11"/>
+      <c r="B83" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C83" s="5"/>
-      <c r="D83" s="3"/>
-      <c r="E83" s="43"/>
-      <c r="F83" s="7"/>
+      <c r="D83" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E83" s="43">
+        <v>184</v>
+      </c>
+      <c r="F83" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="84" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B84" s="11"/>
+      <c r="B84" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C84" s="5"/>
-      <c r="D84" s="3"/>
-      <c r="E84" s="43"/>
-      <c r="F84" s="7"/>
+      <c r="D84" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E84" s="43">
+        <v>1884.84</v>
+      </c>
+      <c r="F84" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="85" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B85" s="11"/>
+      <c r="B85" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C85" s="5"/>
-      <c r="D85" s="3"/>
-      <c r="E85" s="43"/>
-      <c r="F85" s="7"/>
+      <c r="D85" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E85" s="43">
+        <v>165</v>
+      </c>
+      <c r="F85" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="86" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B86" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-02 08:16
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1524" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{541D4054-AF43-4099-8FA6-0B4EFEEDB118}"/>
+  <xr:revisionPtr revIDLastSave="1545" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{150FDE29-9113-41D6-B06B-474907414F11}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2329" uniqueCount="147">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2339" uniqueCount="148">
   <si>
     <t>Custo</t>
   </si>
@@ -482,6 +482,9 @@
   </si>
   <si>
     <t>PNEUS</t>
+  </si>
+  <si>
+    <t>NOVA FREIOS E PEÇAS</t>
   </si>
 </sst>
 </file>
@@ -40815,39 +40818,79 @@
       </c>
     </row>
     <row r="86" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B86" s="11"/>
+      <c r="B86" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C86" s="5"/>
-      <c r="D86" s="3"/>
-      <c r="E86" s="43"/>
-      <c r="F86" s="7"/>
+      <c r="D86" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E86" s="43">
+        <v>1182</v>
+      </c>
+      <c r="F86" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="87" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B87" s="11"/>
+      <c r="B87" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C87" s="5"/>
-      <c r="D87" s="3"/>
-      <c r="E87" s="43"/>
-      <c r="F87" s="7"/>
+      <c r="D87" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E87" s="43">
+        <v>117.41</v>
+      </c>
+      <c r="F87" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="88" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B88" s="11"/>
+      <c r="B88" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C88" s="5"/>
-      <c r="D88" s="3"/>
-      <c r="E88" s="43"/>
-      <c r="F88" s="7"/>
+      <c r="D88" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E88" s="43">
+        <v>600</v>
+      </c>
+      <c r="F88" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="89" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B89" s="11"/>
+      <c r="B89" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C89" s="5"/>
-      <c r="D89" s="3"/>
-      <c r="E89" s="43"/>
-      <c r="F89" s="7"/>
+      <c r="D89" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E89" s="43">
+        <v>402</v>
+      </c>
+      <c r="F89" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="90" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B90" s="11"/>
+      <c r="B90" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C90" s="5"/>
-      <c r="D90" s="3"/>
-      <c r="E90" s="43"/>
-      <c r="F90" s="7"/>
+      <c r="D90" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E90" s="43">
+        <v>902.1</v>
+      </c>
+      <c r="F90" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="91" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B91" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-02 12:52
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1545" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{150FDE29-9113-41D6-B06B-474907414F11}"/>
+  <xr:revisionPtr revIDLastSave="1596" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9297217F-0015-4D63-8416-76ADD9900227}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2339" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2357" uniqueCount="149">
   <si>
     <t>Custo</t>
   </si>
@@ -485,6 +485,9 @@
   </si>
   <si>
     <t>NOVA FREIOS E PEÇAS</t>
+  </si>
+  <si>
+    <t>PNEUS MAX</t>
   </si>
 </sst>
 </file>
@@ -17352,17 +17355,21 @@
       </c>
     </row>
     <row r="1079" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1079" s="11"/>
+      <c r="B1079" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C1079" s="5"/>
-      <c r="D1079" s="3"/>
-      <c r="E1079" s="19"/>
-      <c r="F1079" s="7"/>
+      <c r="D1079" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E1079" s="19">
+        <v>12600</v>
+      </c>
+      <c r="F1079" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1080" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1080" s="11"/>
-      <c r="C1080" s="5"/>
-      <c r="D1080" s="3"/>
-      <c r="E1080" s="19"/>
       <c r="F1080" s="7"/>
     </row>
     <row r="1081" spans="2:6" x14ac:dyDescent="0.25">
@@ -40893,67 +40900,139 @@
       </c>
     </row>
     <row r="91" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B91" s="11"/>
+      <c r="B91" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C91" s="5"/>
-      <c r="D91" s="3"/>
-      <c r="E91" s="43"/>
-      <c r="F91" s="7"/>
+      <c r="D91" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E91" s="43">
+        <v>3264</v>
+      </c>
+      <c r="F91" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="92" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B92" s="11"/>
+      <c r="B92" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C92" s="5"/>
-      <c r="D92" s="3"/>
-      <c r="E92" s="43"/>
-      <c r="F92" s="7"/>
+      <c r="D92" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E92" s="43">
+        <v>2900</v>
+      </c>
+      <c r="F92" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="93" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B93" s="11"/>
+      <c r="B93" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C93" s="5"/>
-      <c r="D93" s="3"/>
-      <c r="E93" s="43"/>
-      <c r="F93" s="7"/>
+      <c r="D93" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E93" s="43">
+        <v>325</v>
+      </c>
+      <c r="F93" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="94" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B94" s="11"/>
+      <c r="B94" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C94" s="5"/>
-      <c r="D94" s="3"/>
-      <c r="E94" s="43"/>
-      <c r="F94" s="7"/>
+      <c r="D94" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E94" s="19">
+        <v>1260</v>
+      </c>
+      <c r="F94" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="95" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B95" s="11"/>
+      <c r="B95" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C95" s="5"/>
-      <c r="D95" s="3"/>
-      <c r="E95" s="43"/>
-      <c r="F95" s="7"/>
+      <c r="D95" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E95" s="43">
+        <v>3000</v>
+      </c>
+      <c r="F95" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="96" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B96" s="11"/>
+      <c r="B96" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C96" s="5"/>
-      <c r="D96" s="3"/>
-      <c r="E96" s="43"/>
-      <c r="F96" s="7"/>
+      <c r="D96" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E96" s="43">
+        <v>600</v>
+      </c>
+      <c r="F96" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="97" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B97" s="11"/>
-      <c r="C97" s="5"/>
-      <c r="D97" s="3"/>
-      <c r="E97" s="43"/>
-      <c r="F97" s="7"/>
+      <c r="B97" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="C97" s="24"/>
+      <c r="D97" s="24" t="s">
+        <v>42</v>
+      </c>
+      <c r="E97" s="48">
+        <v>518.35</v>
+      </c>
+      <c r="F97" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="98" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B98" s="11"/>
+      <c r="B98" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C98" s="5"/>
-      <c r="D98" s="3"/>
-      <c r="E98" s="43"/>
-      <c r="F98" s="7"/>
+      <c r="D98" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E98" s="43">
+        <v>100</v>
+      </c>
+      <c r="F98" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="99" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B99" s="11"/>
+      <c r="B99" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C99" s="5"/>
-      <c r="D99" s="3"/>
-      <c r="E99" s="43"/>
-      <c r="F99" s="7"/>
+      <c r="D99" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E99" s="43">
+        <v>505</v>
+      </c>
+      <c r="F99" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="100" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B100" s="11"/>
@@ -60863,21 +60942,6 @@
       <c r="E2943" s="48"/>
       <c r="F2943" s="7"/>
     </row>
-    <row r="2944" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2944" s="24" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2944" s="24"/>
-      <c r="D2944" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="E2944" s="48">
-        <v>518.35</v>
-      </c>
-      <c r="F2944" s="7">
-        <v>46023</v>
-      </c>
-    </row>
     <row r="2945" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2945" s="24"/>
       <c r="C2945" s="24"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-09 09:57
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1637" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{241F45C3-221F-4D1C-BC8D-5A9199C92226}"/>
+  <xr:revisionPtr revIDLastSave="1732" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2033DD5B-D805-4547-A370-A9FCA34F733D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2374" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2420" uniqueCount="154">
   <si>
     <t>Custo</t>
   </si>
@@ -500,6 +500,9 @@
   </si>
   <si>
     <t>DALMEIDA</t>
+  </si>
+  <si>
+    <t>DAF SANCAR</t>
   </si>
 </sst>
 </file>
@@ -41166,165 +41169,349 @@
       </c>
     </row>
     <row r="108" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B108" s="11"/>
+      <c r="B108" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C108" s="5"/>
-      <c r="D108" s="3"/>
-      <c r="E108" s="43"/>
-      <c r="F108" s="7"/>
+      <c r="D108" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E108" s="43">
+        <v>400</v>
+      </c>
+      <c r="F108" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="109" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B109" s="11"/>
+      <c r="B109" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C109" s="5"/>
-      <c r="D109" s="3"/>
-      <c r="E109" s="43"/>
-      <c r="F109" s="7"/>
+      <c r="D109" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E109" s="43">
+        <v>30</v>
+      </c>
+      <c r="F109" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="110" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B110" s="11"/>
+      <c r="B110" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C110" s="5"/>
-      <c r="D110" s="3"/>
-      <c r="E110" s="43"/>
-      <c r="F110" s="7"/>
+      <c r="D110" s="3" t="s">
+        <v>153</v>
+      </c>
+      <c r="E110" s="43">
+        <v>2735.31</v>
+      </c>
+      <c r="F110" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="111" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B111" s="11"/>
+      <c r="B111" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C111" s="5"/>
-      <c r="D111" s="3"/>
-      <c r="E111" s="43"/>
-      <c r="F111" s="7"/>
+      <c r="D111" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E111" s="43">
+        <v>100</v>
+      </c>
+      <c r="F111" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="112" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B112" s="11"/>
+      <c r="B112" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C112" s="5"/>
-      <c r="D112" s="3"/>
-      <c r="E112" s="43"/>
-      <c r="F112" s="7"/>
+      <c r="D112" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E112" s="43">
+        <v>1805</v>
+      </c>
+      <c r="F112" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="113" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B113" s="11"/>
+      <c r="B113" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C113" s="5"/>
-      <c r="D113" s="3"/>
-      <c r="E113" s="43"/>
-      <c r="F113" s="7"/>
+      <c r="D113" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E113" s="43">
+        <v>200</v>
+      </c>
+      <c r="F113" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="114" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B114" s="11"/>
+      <c r="B114" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C114" s="5"/>
-      <c r="D114" s="3"/>
-      <c r="E114" s="43"/>
-      <c r="F114" s="7"/>
+      <c r="D114" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E114" s="43">
+        <v>90</v>
+      </c>
+      <c r="F114" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="115" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B115" s="11"/>
+      <c r="B115" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C115" s="5"/>
-      <c r="D115" s="3"/>
-      <c r="E115" s="43"/>
-      <c r="F115" s="7"/>
+      <c r="D115" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E115" s="43">
+        <v>642.5</v>
+      </c>
+      <c r="F115" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="116" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B116" s="11"/>
+      <c r="B116" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C116" s="5"/>
-      <c r="D116" s="3"/>
-      <c r="E116" s="43"/>
-      <c r="F116" s="7"/>
+      <c r="D116" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E116" s="43">
+        <v>930</v>
+      </c>
+      <c r="F116" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="117" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B117" s="11"/>
+      <c r="B117" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C117" s="5"/>
-      <c r="D117" s="3"/>
-      <c r="E117" s="43"/>
-      <c r="F117" s="7"/>
+      <c r="D117" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E117" s="43">
+        <v>1285</v>
+      </c>
+      <c r="F117" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="118" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B118" s="11"/>
+      <c r="B118" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C118" s="5"/>
-      <c r="D118" s="3"/>
-      <c r="E118" s="43"/>
-      <c r="F118" s="7"/>
+      <c r="D118" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E118" s="43">
+        <v>430</v>
+      </c>
+      <c r="F118" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="119" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B119" s="11"/>
+      <c r="B119" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C119" s="5"/>
-      <c r="D119" s="3"/>
-      <c r="E119" s="43"/>
-      <c r="F119" s="7"/>
+      <c r="D119" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E119" s="43">
+        <v>2458.4</v>
+      </c>
+      <c r="F119" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="120" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B120" s="11"/>
+      <c r="B120" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C120" s="5"/>
-      <c r="D120" s="3"/>
-      <c r="E120" s="43"/>
-      <c r="F120" s="7"/>
+      <c r="D120" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E120" s="43">
+        <v>500</v>
+      </c>
+      <c r="F120" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="121" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B121" s="11"/>
+      <c r="B121" s="11" t="s">
+        <v>124</v>
+      </c>
       <c r="C121" s="5"/>
-      <c r="D121" s="3"/>
-      <c r="E121" s="43"/>
-      <c r="F121" s="7"/>
+      <c r="D121" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E121" s="43">
+        <v>425</v>
+      </c>
+      <c r="F121" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="122" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B122" s="11"/>
+      <c r="B122" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C122" s="5"/>
-      <c r="D122" s="3"/>
-      <c r="E122" s="43"/>
-      <c r="F122" s="7"/>
+      <c r="D122" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E122" s="43">
+        <v>2930</v>
+      </c>
+      <c r="F122" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="123" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B123" s="11"/>
+      <c r="B123" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C123" s="5"/>
-      <c r="D123" s="3"/>
-      <c r="E123" s="43"/>
-      <c r="F123" s="7"/>
+      <c r="D123" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E123" s="43">
+        <v>70</v>
+      </c>
+      <c r="F123" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="124" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B124" s="11"/>
+      <c r="B124" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C124" s="5"/>
-      <c r="D124" s="3"/>
-      <c r="E124" s="43"/>
-      <c r="F124" s="7"/>
+      <c r="D124" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E124" s="43">
+        <v>200</v>
+      </c>
+      <c r="F124" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="125" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B125" s="11"/>
+      <c r="B125" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C125" s="5"/>
-      <c r="D125" s="3"/>
-      <c r="E125" s="43"/>
-      <c r="F125" s="7"/>
+      <c r="D125" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E125" s="43">
+        <v>700</v>
+      </c>
+      <c r="F125" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="126" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B126" s="11"/>
+      <c r="B126" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C126" s="5"/>
-      <c r="D126" s="3"/>
-      <c r="E126" s="43"/>
-      <c r="F126" s="7"/>
+      <c r="D126" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E126" s="43">
+        <v>1300</v>
+      </c>
+      <c r="F126" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="127" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B127" s="11"/>
+      <c r="B127" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C127" s="5"/>
-      <c r="D127" s="3"/>
-      <c r="E127" s="43"/>
-      <c r="F127" s="7"/>
+      <c r="D127" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E127" s="43">
+        <v>1100</v>
+      </c>
+      <c r="F127" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="128" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B128" s="11"/>
+      <c r="B128" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C128" s="5"/>
-      <c r="D128" s="3"/>
-      <c r="E128" s="43"/>
-      <c r="F128" s="7"/>
+      <c r="D128" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E128" s="43">
+        <v>1287</v>
+      </c>
+      <c r="F128" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="129" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B129" s="11"/>
+      <c r="B129" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C129" s="5"/>
-      <c r="D129" s="3"/>
-      <c r="E129" s="43"/>
-      <c r="F129" s="7"/>
+      <c r="D129" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E129" s="43">
+        <v>805.5</v>
+      </c>
+      <c r="F129" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="130" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B130" s="11"/>
+      <c r="B130" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C130" s="5"/>
-      <c r="D130" s="3"/>
-      <c r="E130" s="43"/>
-      <c r="F130" s="7"/>
+      <c r="D130" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E130" s="43">
+        <v>43</v>
+      </c>
+      <c r="F130" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="131" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B131" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-09 13:03
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1732" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2033DD5B-D805-4547-A370-A9FCA34F733D}"/>
+  <xr:revisionPtr revIDLastSave="1737" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{029E7EF9-91B9-43C9-A4CC-A3B6E9C2622C}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2420" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2422" uniqueCount="154">
   <si>
     <t>Custo</t>
   </si>
@@ -41514,11 +41514,19 @@
       </c>
     </row>
     <row r="131" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B131" s="11"/>
+      <c r="B131" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="C131" s="5"/>
-      <c r="D131" s="3"/>
-      <c r="E131" s="43"/>
-      <c r="F131" s="7"/>
+      <c r="D131" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E131" s="43">
+        <v>214</v>
+      </c>
+      <c r="F131" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="132" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B132" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-11 09:06
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1737" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{029E7EF9-91B9-43C9-A4CC-A3B6E9C2622C}"/>
+  <xr:revisionPtr revIDLastSave="1840" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BB0A405-1C76-4FE2-A563-9E698248BE50}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2422" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2474" uniqueCount="155">
   <si>
     <t>Custo</t>
   </si>
@@ -503,6 +503,9 @@
   </si>
   <si>
     <t>DAF SANCAR</t>
+  </si>
+  <si>
+    <t>SILVA CARROCERIA</t>
   </si>
 </sst>
 </file>
@@ -41529,186 +41532,394 @@
       </c>
     </row>
     <row r="132" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B132" s="11"/>
+      <c r="B132" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C132" s="5"/>
-      <c r="D132" s="3"/>
-      <c r="E132" s="43"/>
-      <c r="F132" s="7"/>
+      <c r="D132" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E132" s="43">
+        <v>95</v>
+      </c>
+      <c r="F132" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="133" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B133" s="11"/>
+      <c r="B133" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C133" s="5"/>
-      <c r="D133" s="3"/>
-      <c r="E133" s="43"/>
-      <c r="F133" s="7"/>
+      <c r="D133" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E133" s="43">
+        <v>360</v>
+      </c>
+      <c r="F133" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="134" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B134" s="11"/>
+      <c r="B134" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C134" s="5"/>
-      <c r="D134" s="3"/>
-      <c r="E134" s="43"/>
-      <c r="F134" s="7"/>
+      <c r="D134" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E134" s="43">
+        <v>310</v>
+      </c>
+      <c r="F134" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="135" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B135" s="11"/>
+      <c r="B135" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C135" s="5"/>
-      <c r="D135" s="3"/>
-      <c r="E135" s="43"/>
-      <c r="F135" s="7"/>
+      <c r="D135" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E135" s="43">
+        <v>1350</v>
+      </c>
+      <c r="F135" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="136" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B136" s="11"/>
+      <c r="B136" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C136" s="5"/>
-      <c r="D136" s="3"/>
-      <c r="E136" s="43"/>
-      <c r="F136" s="7"/>
+      <c r="D136" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E136" s="43">
+        <v>190</v>
+      </c>
+      <c r="F136" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="137" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B137" s="11"/>
+      <c r="B137" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C137" s="5"/>
-      <c r="D137" s="3"/>
-      <c r="E137" s="43"/>
-      <c r="F137" s="7"/>
+      <c r="D137" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E137" s="43">
+        <v>720</v>
+      </c>
+      <c r="F137" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="138" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B138" s="11"/>
+      <c r="B138" s="11" t="s">
+        <v>142</v>
+      </c>
       <c r="C138" s="5"/>
-      <c r="D138" s="3"/>
-      <c r="E138" s="43"/>
-      <c r="F138" s="7"/>
+      <c r="D138" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E138" s="43">
+        <v>160</v>
+      </c>
+      <c r="F138" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="139" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B139" s="11"/>
+      <c r="B139" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C139" s="5"/>
-      <c r="D139" s="3"/>
-      <c r="E139" s="43"/>
-      <c r="F139" s="7"/>
+      <c r="D139" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E139" s="43">
+        <v>180</v>
+      </c>
+      <c r="F139" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="140" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B140" s="11"/>
+      <c r="B140" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C140" s="5"/>
-      <c r="D140" s="3"/>
-      <c r="E140" s="43"/>
-      <c r="F140" s="7"/>
+      <c r="D140" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="E140" s="43">
+        <v>2710</v>
+      </c>
+      <c r="F140" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="141" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B141" s="11"/>
+      <c r="B141" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C141" s="5"/>
-      <c r="D141" s="3"/>
-      <c r="E141" s="43"/>
-      <c r="F141" s="7"/>
+      <c r="D141" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E141" s="43">
+        <v>920</v>
+      </c>
+      <c r="F141" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="142" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B142" s="11"/>
+      <c r="B142" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C142" s="5"/>
-      <c r="D142" s="3"/>
-      <c r="E142" s="43"/>
-      <c r="F142" s="7"/>
+      <c r="D142" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E142" s="43">
+        <v>40</v>
+      </c>
+      <c r="F142" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="143" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B143" s="11"/>
+      <c r="B143" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C143" s="5"/>
-      <c r="D143" s="3"/>
-      <c r="E143" s="43"/>
-      <c r="F143" s="7"/>
+      <c r="D143" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E143" s="43">
+        <v>390</v>
+      </c>
+      <c r="F143" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="144" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B144" s="11"/>
+      <c r="B144" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C144" s="5"/>
-      <c r="D144" s="3"/>
-      <c r="E144" s="43"/>
-      <c r="F144" s="7"/>
+      <c r="D144" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E144" s="43">
+        <v>70</v>
+      </c>
+      <c r="F144" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="145" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B145" s="11"/>
+      <c r="B145" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C145" s="5"/>
-      <c r="D145" s="3"/>
-      <c r="E145" s="43"/>
-      <c r="F145" s="7"/>
+      <c r="D145" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E145" s="43">
+        <v>200</v>
+      </c>
+      <c r="F145" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="146" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B146" s="11"/>
+      <c r="B146" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C146" s="5"/>
-      <c r="D146" s="3"/>
-      <c r="E146" s="43"/>
-      <c r="F146" s="7"/>
+      <c r="D146" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E146" s="43">
+        <v>1083.3</v>
+      </c>
+      <c r="F146" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="147" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B147" s="11"/>
+      <c r="B147" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C147" s="5"/>
-      <c r="D147" s="3"/>
-      <c r="E147" s="43"/>
-      <c r="F147" s="7"/>
+      <c r="D147" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E147" s="43">
+        <v>100</v>
+      </c>
+      <c r="F147" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="148" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B148" s="11"/>
+      <c r="B148" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C148" s="5"/>
-      <c r="D148" s="3"/>
-      <c r="E148" s="43"/>
-      <c r="F148" s="7"/>
+      <c r="D148" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E148" s="43">
+        <v>1500</v>
+      </c>
+      <c r="F148" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="149" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B149" s="11"/>
+      <c r="B149" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C149" s="5"/>
-      <c r="D149" s="3"/>
-      <c r="E149" s="43"/>
-      <c r="F149" s="7"/>
+      <c r="D149" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E149" s="43">
+        <v>35</v>
+      </c>
+      <c r="F149" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="150" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B150" s="11"/>
+      <c r="B150" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C150" s="5"/>
-      <c r="D150" s="3"/>
-      <c r="E150" s="43"/>
-      <c r="F150" s="7"/>
+      <c r="D150" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E150" s="43">
+        <v>120</v>
+      </c>
+      <c r="F150" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="151" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B151" s="11"/>
+      <c r="B151" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C151" s="5"/>
-      <c r="D151" s="3"/>
-      <c r="E151" s="43"/>
-      <c r="F151" s="7"/>
+      <c r="D151" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E151" s="43">
+        <v>65</v>
+      </c>
+      <c r="F151" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="152" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B152" s="11"/>
+      <c r="B152" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C152" s="5"/>
-      <c r="D152" s="3"/>
-      <c r="E152" s="43"/>
-      <c r="F152" s="7"/>
+      <c r="D152" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E152" s="43">
+        <v>50</v>
+      </c>
+      <c r="F152" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="153" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B153" s="11"/>
+      <c r="B153" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C153" s="5"/>
-      <c r="D153" s="3"/>
-      <c r="E153" s="43"/>
-      <c r="F153" s="7"/>
+      <c r="D153" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E153" s="43">
+        <v>343</v>
+      </c>
+      <c r="F153" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="154" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B154" s="11"/>
+      <c r="B154" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C154" s="5"/>
-      <c r="D154" s="3"/>
-      <c r="E154" s="43"/>
-      <c r="F154" s="7"/>
+      <c r="D154" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E154" s="43">
+        <v>1339</v>
+      </c>
+      <c r="F154" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="155" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B155" s="11"/>
+      <c r="B155" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C155" s="5"/>
-      <c r="D155" s="3"/>
-      <c r="E155" s="43"/>
-      <c r="F155" s="7"/>
+      <c r="D155" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E155" s="43">
+        <v>150</v>
+      </c>
+      <c r="F155" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="156" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B156" s="11"/>
+      <c r="B156" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C156" s="5"/>
-      <c r="D156" s="3"/>
-      <c r="E156" s="43"/>
-      <c r="F156" s="7"/>
+      <c r="D156" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E156" s="43">
+        <v>606</v>
+      </c>
+      <c r="F156" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="157" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B157" s="11"/>
+      <c r="B157" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C157" s="5"/>
-      <c r="D157" s="3"/>
-      <c r="E157" s="43"/>
-      <c r="F157" s="7"/>
+      <c r="D157" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E157" s="43">
+        <v>100</v>
+      </c>
+      <c r="F157" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="158" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B158" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-13 08:39
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1840" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8BB0A405-1C76-4FE2-A563-9E698248BE50}"/>
+  <xr:revisionPtr revIDLastSave="1867" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98D2DBEE-BCCF-4A7A-AE23-F8D92B52D14D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2474" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2490" uniqueCount="157">
   <si>
     <t>Custo</t>
   </si>
@@ -506,6 +506,12 @@
   </si>
   <si>
     <t>SILVA CARROCERIA</t>
+  </si>
+  <si>
+    <t>PNEU MAX</t>
+  </si>
+  <si>
+    <t>BORRACHARIA NITEROI</t>
   </si>
 </sst>
 </file>
@@ -41922,60 +41928,124 @@
       </c>
     </row>
     <row r="158" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B158" s="11"/>
+      <c r="B158" s="11" t="s">
+        <v>31</v>
+      </c>
       <c r="C158" s="5"/>
-      <c r="D158" s="3"/>
-      <c r="E158" s="43"/>
-      <c r="F158" s="7"/>
+      <c r="D158" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E158" s="43">
+        <v>280</v>
+      </c>
+      <c r="F158" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="159" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B159" s="11"/>
+      <c r="B159" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C159" s="5"/>
-      <c r="D159" s="3"/>
-      <c r="E159" s="43"/>
-      <c r="F159" s="7"/>
+      <c r="D159" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E159" s="43">
+        <v>1508</v>
+      </c>
+      <c r="F159" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="160" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B160" s="11"/>
+      <c r="B160" s="11" t="s">
+        <v>31</v>
+      </c>
       <c r="C160" s="5"/>
-      <c r="D160" s="3"/>
-      <c r="E160" s="43"/>
-      <c r="F160" s="7"/>
+      <c r="D160" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E160" s="43">
+        <v>67</v>
+      </c>
+      <c r="F160" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="161" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B161" s="11"/>
+      <c r="B161" s="11" t="s">
+        <v>31</v>
+      </c>
       <c r="C161" s="5"/>
-      <c r="D161" s="3"/>
-      <c r="E161" s="43"/>
-      <c r="F161" s="7"/>
+      <c r="D161" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E161" s="43">
+        <v>30</v>
+      </c>
+      <c r="F161" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="162" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B162" s="11"/>
+      <c r="B162" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C162" s="5"/>
-      <c r="D162" s="3"/>
-      <c r="E162" s="43"/>
-      <c r="F162" s="7"/>
+      <c r="D162" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E162" s="43">
+        <v>3635</v>
+      </c>
+      <c r="F162" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="163" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B163" s="11"/>
+      <c r="B163" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C163" s="5"/>
-      <c r="D163" s="3"/>
-      <c r="E163" s="43"/>
-      <c r="F163" s="7"/>
+      <c r="D163" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E163" s="43">
+        <v>4200</v>
+      </c>
+      <c r="F163" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="164" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B164" s="11"/>
+      <c r="B164" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C164" s="5"/>
-      <c r="D164" s="3"/>
-      <c r="E164" s="43"/>
-      <c r="F164" s="7"/>
+      <c r="D164" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E164" s="43">
+        <v>1497</v>
+      </c>
+      <c r="F164" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="165" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B165" s="11"/>
+      <c r="B165" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C165" s="5"/>
-      <c r="D165" s="3"/>
-      <c r="E165" s="43"/>
-      <c r="F165" s="7"/>
+      <c r="D165" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E165" s="43">
+        <v>2944</v>
+      </c>
+      <c r="F165" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="166" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B166" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-18 10:19
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1867" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{98D2DBEE-BCCF-4A7A-AE23-F8D92B52D14D}"/>
+  <xr:revisionPtr revIDLastSave="1897" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A0F3D02-81E1-4ECD-8884-A9490C15A990}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2490" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="158">
   <si>
     <t>Custo</t>
   </si>
@@ -512,6 +512,9 @@
   </si>
   <si>
     <t>BORRACHARIA NITEROI</t>
+  </si>
+  <si>
+    <t>TEQ5C84</t>
   </si>
 </sst>
 </file>
@@ -42048,53 +42051,109 @@
       </c>
     </row>
     <row r="166" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B166" s="11"/>
+      <c r="B166" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C166" s="5"/>
-      <c r="D166" s="3"/>
-      <c r="E166" s="43"/>
-      <c r="F166" s="7"/>
+      <c r="D166" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E166" s="43">
+        <v>122</v>
+      </c>
+      <c r="F166" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="167" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B167" s="11"/>
+      <c r="B167" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C167" s="5"/>
-      <c r="D167" s="3"/>
-      <c r="E167" s="43"/>
-      <c r="F167" s="7"/>
+      <c r="D167" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E167" s="43">
+        <v>40</v>
+      </c>
+      <c r="F167" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="168" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B168" s="11"/>
+      <c r="B168" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C168" s="5"/>
-      <c r="D168" s="3"/>
-      <c r="E168" s="43"/>
-      <c r="F168" s="7"/>
+      <c r="D168" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E168" s="43">
+        <v>100</v>
+      </c>
+      <c r="F168" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="169" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B169" s="11"/>
+      <c r="B169" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C169" s="5"/>
-      <c r="D169" s="3"/>
-      <c r="E169" s="43"/>
-      <c r="F169" s="7"/>
+      <c r="D169" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E169" s="43">
+        <v>50</v>
+      </c>
+      <c r="F169" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="170" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B170" s="11"/>
+      <c r="B170" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C170" s="5"/>
-      <c r="D170" s="3"/>
-      <c r="E170" s="43"/>
-      <c r="F170" s="7"/>
+      <c r="D170" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E170" s="43">
+        <v>12</v>
+      </c>
+      <c r="F170" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="171" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B171" s="11"/>
+      <c r="B171" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="C171" s="5"/>
-      <c r="D171" s="3"/>
-      <c r="E171" s="43"/>
-      <c r="F171" s="7"/>
+      <c r="D171" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E171" s="43">
+        <v>210</v>
+      </c>
+      <c r="F171" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="172" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B172" s="11"/>
+      <c r="B172" s="11" t="s">
+        <v>157</v>
+      </c>
       <c r="C172" s="5"/>
-      <c r="D172" s="3"/>
-      <c r="E172" s="43"/>
-      <c r="F172" s="7"/>
+      <c r="D172" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E172" s="43">
+        <v>55</v>
+      </c>
+      <c r="F172" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="173" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B173" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-18 11:50
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1897" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A0F3D02-81E1-4ECD-8884-A9490C15A990}"/>
+  <xr:revisionPtr revIDLastSave="1905" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34BE65B4-AA1B-446F-A968-3FC4FC7D3240}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2504" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2508" uniqueCount="158">
   <si>
     <t>Custo</t>
   </si>
@@ -42156,18 +42156,34 @@
       </c>
     </row>
     <row r="173" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B173" s="11"/>
+      <c r="B173" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C173" s="5"/>
-      <c r="D173" s="3"/>
-      <c r="E173" s="43"/>
-      <c r="F173" s="7"/>
+      <c r="D173" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E173" s="43">
+        <v>100</v>
+      </c>
+      <c r="F173" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="174" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B174" s="11"/>
+      <c r="B174" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C174" s="5"/>
-      <c r="D174" s="3"/>
-      <c r="E174" s="43"/>
-      <c r="F174" s="7"/>
+      <c r="D174" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E174" s="43">
+        <v>70</v>
+      </c>
+      <c r="F174" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="175" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B175" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-25 16:37
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1905" documentId="8_{99301734-F318-4AB5-A368-7B22515FFAD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{34BE65B4-AA1B-446F-A968-3FC4FC7D3240}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1785F16A-F5B8-4E25-831A-CCA32E76DB98}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2508" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2552" uniqueCount="162">
   <si>
     <t>Custo</t>
   </si>
@@ -515,6 +515,18 @@
   </si>
   <si>
     <t>TEQ5C84</t>
+  </si>
+  <si>
+    <t>OFICINA CATALÃO DIESEL</t>
+  </si>
+  <si>
+    <t>AUTO ESCAPAMENTO FREITAS</t>
+  </si>
+  <si>
+    <t>AUTO PEÇAS DALDEGAN</t>
+  </si>
+  <si>
+    <t>CT DIESEL</t>
   </si>
 </sst>
 </file>
@@ -42186,158 +42198,334 @@
       </c>
     </row>
     <row r="175" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B175" s="11"/>
+      <c r="B175" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C175" s="5"/>
-      <c r="D175" s="3"/>
-      <c r="E175" s="43"/>
-      <c r="F175" s="7"/>
+      <c r="D175" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E175" s="43">
+        <v>1102</v>
+      </c>
+      <c r="F175" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="176" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B176" s="11"/>
+      <c r="B176" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C176" s="5"/>
-      <c r="D176" s="3"/>
-      <c r="E176" s="43"/>
-      <c r="F176" s="7"/>
+      <c r="D176" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E176" s="43">
+        <v>1200</v>
+      </c>
+      <c r="F176" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="177" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B177" s="11"/>
+      <c r="B177" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C177" s="5"/>
-      <c r="D177" s="3"/>
-      <c r="E177" s="43"/>
-      <c r="F177" s="7"/>
+      <c r="D177" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E177" s="43">
+        <v>280</v>
+      </c>
+      <c r="F177" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="178" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B178" s="11"/>
+      <c r="B178" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C178" s="5"/>
-      <c r="D178" s="3"/>
-      <c r="E178" s="43"/>
-      <c r="F178" s="7"/>
+      <c r="D178" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E178" s="43">
+        <v>46</v>
+      </c>
+      <c r="F178" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="179" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B179" s="11"/>
+      <c r="B179" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C179" s="5"/>
-      <c r="D179" s="3"/>
-      <c r="E179" s="43"/>
-      <c r="F179" s="7"/>
+      <c r="D179" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E179" s="43">
+        <v>136.9</v>
+      </c>
+      <c r="F179" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="180" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B180" s="11"/>
+      <c r="B180" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C180" s="5"/>
-      <c r="D180" s="3"/>
-      <c r="E180" s="43"/>
-      <c r="F180" s="7"/>
+      <c r="D180" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E180" s="43">
+        <v>965</v>
+      </c>
+      <c r="F180" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="181" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B181" s="11"/>
+      <c r="B181" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C181" s="5"/>
-      <c r="D181" s="3"/>
-      <c r="E181" s="43"/>
-      <c r="F181" s="7"/>
+      <c r="D181" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E181" s="43">
+        <v>1623.4</v>
+      </c>
+      <c r="F181" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="182" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B182" s="11"/>
+      <c r="B182" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C182" s="5"/>
-      <c r="D182" s="3"/>
-      <c r="E182" s="43"/>
-      <c r="F182" s="7"/>
+      <c r="D182" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E182" s="43">
+        <v>130</v>
+      </c>
+      <c r="F182" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="183" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B183" s="11"/>
+      <c r="B183" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C183" s="5"/>
-      <c r="D183" s="3"/>
-      <c r="E183" s="43"/>
-      <c r="F183" s="7"/>
+      <c r="D183" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E183" s="43">
+        <v>1908</v>
+      </c>
+      <c r="F183" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="184" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B184" s="11"/>
+      <c r="B184" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C184" s="5"/>
-      <c r="D184" s="3"/>
-      <c r="E184" s="43"/>
-      <c r="F184" s="7"/>
+      <c r="D184" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E184" s="43">
+        <v>1435</v>
+      </c>
+      <c r="F184" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="185" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B185" s="11"/>
+      <c r="B185" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C185" s="5"/>
-      <c r="D185" s="3"/>
-      <c r="E185" s="43"/>
-      <c r="F185" s="7"/>
+      <c r="D185" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E185" s="43">
+        <v>224.18</v>
+      </c>
+      <c r="F185" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="186" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B186" s="11"/>
+      <c r="B186" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C186" s="5"/>
-      <c r="D186" s="3"/>
-      <c r="E186" s="43"/>
-      <c r="F186" s="7"/>
+      <c r="D186" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E186" s="43">
+        <v>100</v>
+      </c>
+      <c r="F186" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="187" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B187" s="11"/>
+      <c r="B187" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C187" s="5"/>
-      <c r="D187" s="3"/>
-      <c r="E187" s="43"/>
-      <c r="F187" s="7"/>
+      <c r="D187" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E187" s="43">
+        <v>250</v>
+      </c>
+      <c r="F187" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="188" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B188" s="11"/>
+      <c r="B188" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C188" s="5"/>
-      <c r="D188" s="3"/>
-      <c r="E188" s="43"/>
-      <c r="F188" s="7"/>
+      <c r="D188" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E188" s="43">
+        <v>135</v>
+      </c>
+      <c r="F188" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="189" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B189" s="11"/>
+      <c r="B189" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C189" s="5"/>
-      <c r="D189" s="3"/>
-      <c r="E189" s="43"/>
-      <c r="F189" s="7"/>
+      <c r="D189" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E189" s="43">
+        <v>855</v>
+      </c>
+      <c r="F189" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="190" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B190" s="11"/>
+      <c r="B190" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C190" s="5"/>
-      <c r="D190" s="3"/>
-      <c r="E190" s="43"/>
-      <c r="F190" s="7"/>
+      <c r="D190" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E190" s="43">
+        <v>280</v>
+      </c>
+      <c r="F190" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="191" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B191" s="11"/>
+      <c r="B191" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C191" s="5"/>
-      <c r="D191" s="3"/>
-      <c r="E191" s="43"/>
-      <c r="F191" s="7"/>
+      <c r="D191" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E191" s="43">
+        <v>1700</v>
+      </c>
+      <c r="F191" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="192" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B192" s="11"/>
+      <c r="B192" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C192" s="5"/>
-      <c r="D192" s="3"/>
-      <c r="E192" s="43"/>
-      <c r="F192" s="7"/>
+      <c r="D192" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E192" s="43">
+        <v>5576.47</v>
+      </c>
+      <c r="F192" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="193" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B193" s="11"/>
+      <c r="B193" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C193" s="5"/>
-      <c r="D193" s="3"/>
-      <c r="E193" s="43"/>
-      <c r="F193" s="7"/>
+      <c r="D193" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E193" s="43">
+        <v>185.5</v>
+      </c>
+      <c r="F193" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="194" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B194" s="11"/>
+      <c r="B194" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C194" s="5"/>
-      <c r="D194" s="3"/>
-      <c r="E194" s="43"/>
-      <c r="F194" s="7"/>
+      <c r="D194" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E194" s="43">
+        <v>80</v>
+      </c>
+      <c r="F194" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="195" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B195" s="11"/>
+      <c r="B195" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C195" s="5"/>
-      <c r="D195" s="3"/>
-      <c r="E195" s="43"/>
-      <c r="F195" s="7"/>
+      <c r="D195" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E195" s="43">
+        <v>134</v>
+      </c>
+      <c r="F195" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="196" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B196" s="11"/>
+      <c r="B196" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C196" s="5"/>
-      <c r="D196" s="3"/>
-      <c r="E196" s="43"/>
-      <c r="F196" s="7"/>
+      <c r="D196" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E196" s="43">
+        <v>200</v>
+      </c>
+      <c r="F196" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="197" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B197" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-02-26 16:06
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1785F16A-F5B8-4E25-831A-CCA32E76DB98}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C57B275A-21D9-4049-9D63-8AB7635DA7AC}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2552" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2574" uniqueCount="165">
   <si>
     <t>Custo</t>
   </si>
@@ -527,6 +527,15 @@
   </si>
   <si>
     <t>CT DIESEL</t>
+  </si>
+  <si>
+    <t>OFICINA DO RODINHO</t>
+  </si>
+  <si>
+    <t>KLM TRANSPORTES</t>
+  </si>
+  <si>
+    <t>HMR9D08</t>
   </si>
 </sst>
 </file>
@@ -42528,81 +42537,169 @@
       </c>
     </row>
     <row r="197" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B197" s="11"/>
+      <c r="B197" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C197" s="5"/>
-      <c r="D197" s="3"/>
-      <c r="E197" s="43"/>
-      <c r="F197" s="7"/>
+      <c r="D197" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E197" s="43">
+        <v>153</v>
+      </c>
+      <c r="F197" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="198" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B198" s="11"/>
+      <c r="B198" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C198" s="5"/>
-      <c r="D198" s="3"/>
-      <c r="E198" s="43"/>
-      <c r="F198" s="7"/>
+      <c r="D198" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E198" s="43">
+        <v>200</v>
+      </c>
+      <c r="F198" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="199" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B199" s="11"/>
+      <c r="B199" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C199" s="5"/>
-      <c r="D199" s="3"/>
-      <c r="E199" s="43"/>
-      <c r="F199" s="7"/>
+      <c r="D199" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="E199" s="43">
+        <v>150</v>
+      </c>
+      <c r="F199" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="200" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B200" s="11"/>
+      <c r="B200" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C200" s="5"/>
-      <c r="D200" s="3"/>
-      <c r="E200" s="43"/>
-      <c r="F200" s="7"/>
+      <c r="D200" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E200" s="43">
+        <v>1300</v>
+      </c>
+      <c r="F200" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="201" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B201" s="11"/>
+      <c r="B201" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C201" s="5"/>
-      <c r="D201" s="3"/>
-      <c r="E201" s="43"/>
-      <c r="F201" s="7"/>
+      <c r="D201" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E201" s="43">
+        <v>240</v>
+      </c>
+      <c r="F201" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="202" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B202" s="11"/>
+      <c r="B202" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C202" s="5"/>
-      <c r="D202" s="3"/>
-      <c r="E202" s="43"/>
-      <c r="F202" s="7"/>
+      <c r="D202" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E202" s="43">
+        <v>2026.6</v>
+      </c>
+      <c r="F202" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="203" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B203" s="11"/>
+      <c r="B203" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C203" s="5"/>
-      <c r="D203" s="3"/>
-      <c r="E203" s="43"/>
-      <c r="F203" s="7"/>
+      <c r="D203" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E203" s="43">
+        <v>1465.8</v>
+      </c>
+      <c r="F203" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="204" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B204" s="11"/>
+      <c r="B204" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C204" s="5"/>
-      <c r="D204" s="3"/>
-      <c r="E204" s="43"/>
-      <c r="F204" s="7"/>
+      <c r="D204" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E204" s="43">
+        <v>100</v>
+      </c>
+      <c r="F204" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="205" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B205" s="11"/>
+      <c r="B205" s="11" t="s">
+        <v>142</v>
+      </c>
       <c r="C205" s="5"/>
-      <c r="D205" s="3"/>
-      <c r="E205" s="43"/>
-      <c r="F205" s="7"/>
+      <c r="D205" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E205" s="43">
+        <v>612.5</v>
+      </c>
+      <c r="F205" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="206" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B206" s="11"/>
+      <c r="B206" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C206" s="5"/>
-      <c r="D206" s="3"/>
-      <c r="E206" s="43"/>
-      <c r="F206" s="7"/>
+      <c r="D206" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E206" s="43">
+        <v>80</v>
+      </c>
+      <c r="F206" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="207" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B207" s="11"/>
+      <c r="B207" s="11" t="s">
+        <v>164</v>
+      </c>
       <c r="C207" s="5"/>
-      <c r="D207" s="3"/>
-      <c r="E207" s="43"/>
-      <c r="F207" s="7"/>
+      <c r="D207" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E207" s="43">
+        <v>35</v>
+      </c>
+      <c r="F207" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="208" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B208" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-03 13:00
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C57B275A-21D9-4049-9D63-8AB7635DA7AC}"/>
+  <xr:revisionPtr revIDLastSave="98" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02FF2DBB-C695-46F2-B7D3-B2EECCA0E8C3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'2025'!$B$2:$G$4196</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026'!$B$2:$G$2944</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026'!$B$2:$G$2946</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2574" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2590" uniqueCount="167">
   <si>
     <t>Custo</t>
   </si>
@@ -536,6 +536,12 @@
   </si>
   <si>
     <t>HMR9D08</t>
+  </si>
+  <si>
+    <t>JOK PNEUS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BORRACHARIA  </t>
   </si>
 </sst>
 </file>
@@ -42702,46 +42708,94 @@
       </c>
     </row>
     <row r="208" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B208" s="11"/>
+      <c r="B208" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C208" s="5"/>
-      <c r="D208" s="3"/>
-      <c r="E208" s="43"/>
-      <c r="F208" s="7"/>
+      <c r="D208" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E208" s="43">
+        <v>50</v>
+      </c>
+      <c r="F208" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="209" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B209" s="11"/>
+      <c r="B209" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C209" s="5"/>
-      <c r="D209" s="3"/>
-      <c r="E209" s="43"/>
-      <c r="F209" s="7"/>
+      <c r="D209" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E209" s="43">
+        <v>726.9</v>
+      </c>
+      <c r="F209" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="210" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B210" s="11"/>
+      <c r="B210" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C210" s="5"/>
-      <c r="D210" s="3"/>
-      <c r="E210" s="43"/>
-      <c r="F210" s="7"/>
+      <c r="D210" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E210" s="43">
+        <v>50</v>
+      </c>
+      <c r="F210" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="211" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B211" s="11"/>
+      <c r="B211" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C211" s="5"/>
-      <c r="D211" s="3"/>
-      <c r="E211" s="43"/>
-      <c r="F211" s="7"/>
+      <c r="D211" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E211" s="43">
+        <v>140</v>
+      </c>
+      <c r="F211" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="212" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B212" s="11"/>
+      <c r="B212" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C212" s="5"/>
-      <c r="D212" s="3"/>
-      <c r="E212" s="43"/>
-      <c r="F212" s="7"/>
+      <c r="D212" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="E212" s="43">
+        <v>100</v>
+      </c>
+      <c r="F212" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="213" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B213" s="11"/>
+      <c r="B213" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C213" s="5"/>
-      <c r="D213" s="3"/>
-      <c r="E213" s="43"/>
-      <c r="F213" s="7"/>
+      <c r="D213" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E213" s="43">
+        <v>3980</v>
+      </c>
+      <c r="F213" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="214" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B214" s="11"/>
@@ -61854,18 +61908,34 @@
       <c r="F2943" s="7"/>
     </row>
     <row r="2945" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2945" s="24"/>
+      <c r="B2945" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C2945" s="24"/>
-      <c r="D2945" s="24"/>
-      <c r="E2945" s="46"/>
-      <c r="F2945" s="38"/>
+      <c r="D2945" s="24" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2945" s="46">
+        <v>40</v>
+      </c>
+      <c r="F2945" s="7">
+        <v>46023</v>
+      </c>
     </row>
     <row r="2946" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B2946" s="24"/>
+      <c r="B2946" s="24" t="s">
+        <v>3</v>
+      </c>
       <c r="C2946" s="24"/>
-      <c r="D2946" s="24"/>
-      <c r="E2946" s="46"/>
-      <c r="F2946" s="38"/>
+      <c r="D2946" s="24" t="s">
+        <v>98</v>
+      </c>
+      <c r="E2946" s="46">
+        <v>70</v>
+      </c>
+      <c r="F2946" s="38">
+        <v>46054</v>
+      </c>
     </row>
     <row r="2947" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2947" s="24"/>
@@ -62190,7 +62260,7 @@
       <c r="F2992" s="38"/>
     </row>
   </sheetData>
-  <autoFilter ref="B2:G2944" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>
+  <autoFilter ref="B2:G2946" xr:uid="{35CF32DB-1C2A-4D45-8F6F-18BE3AEB45FF}"/>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-03 17:03
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02FF2DBB-C695-46F2-B7D3-B2EECCA0E8C3}"/>
+  <xr:revisionPtr revIDLastSave="105" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ADB41D6-95F4-4504-86AD-18FB3434A5E0}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2590" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2593" uniqueCount="167">
   <si>
     <t>Custo</t>
   </si>
@@ -42798,18 +42798,32 @@
       </c>
     </row>
     <row r="214" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B214" s="11"/>
+      <c r="B214" s="11" t="s">
+        <v>31</v>
+      </c>
       <c r="C214" s="5"/>
-      <c r="D214" s="3"/>
-      <c r="E214" s="43"/>
-      <c r="F214" s="7"/>
+      <c r="D214" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E214" s="43">
+        <v>32</v>
+      </c>
+      <c r="F214" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="215" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B215" s="11"/>
       <c r="C215" s="5"/>
-      <c r="D215" s="3"/>
-      <c r="E215" s="43"/>
-      <c r="F215" s="7"/>
+      <c r="D215" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E215" s="43">
+        <v>550</v>
+      </c>
+      <c r="F215" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="216" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B216" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-16 11:38
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="105" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2ADB41D6-95F4-4504-86AD-18FB3434A5E0}"/>
+  <xr:revisionPtr revIDLastSave="363" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6340FEDA-37CA-457D-B2E0-A5895F5A1E2A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2593" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2718" uniqueCount="172">
   <si>
     <t>Custo</t>
   </si>
@@ -542,6 +542,21 @@
   </si>
   <si>
     <t xml:space="preserve">BORRACHARIA  </t>
+  </si>
+  <si>
+    <t>SEM</t>
+  </si>
+  <si>
+    <t>CARLITO PNEUS</t>
+  </si>
+  <si>
+    <t>TEB9E97</t>
+  </si>
+  <si>
+    <t>VOLKS BEM AUTO PEÇAS</t>
+  </si>
+  <si>
+    <t>MANG DIVI</t>
   </si>
 </sst>
 </file>
@@ -42813,7 +42828,9 @@
       </c>
     </row>
     <row r="215" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B215" s="11"/>
+      <c r="B215" s="11" t="s">
+        <v>167</v>
+      </c>
       <c r="C215" s="5"/>
       <c r="D215" s="3" t="s">
         <v>135</v>
@@ -42826,438 +42843,934 @@
       </c>
     </row>
     <row r="216" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B216" s="11"/>
+      <c r="B216" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C216" s="5"/>
-      <c r="D216" s="3"/>
-      <c r="E216" s="43"/>
-      <c r="F216" s="7"/>
+      <c r="D216" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E216" s="43">
+        <v>420</v>
+      </c>
+      <c r="F216" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="217" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B217" s="11"/>
+      <c r="B217" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C217" s="5"/>
-      <c r="D217" s="3"/>
-      <c r="E217" s="43"/>
-      <c r="F217" s="7"/>
+      <c r="D217" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E217" s="43">
+        <v>2746.74</v>
+      </c>
+      <c r="F217" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="218" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B218" s="11"/>
+      <c r="B218" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C218" s="5"/>
-      <c r="D218" s="3"/>
-      <c r="E218" s="43"/>
-      <c r="F218" s="7"/>
+      <c r="D218" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E218" s="43">
+        <v>72.260000000000005</v>
+      </c>
+      <c r="F218" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="219" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B219" s="11"/>
+      <c r="B219" s="11" t="s">
+        <v>164</v>
+      </c>
       <c r="C219" s="5"/>
-      <c r="D219" s="3"/>
-      <c r="E219" s="43"/>
-      <c r="F219" s="7"/>
+      <c r="D219" s="3" t="s">
+        <v>168</v>
+      </c>
+      <c r="E219" s="43">
+        <v>30</v>
+      </c>
+      <c r="F219" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="220" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B220" s="11"/>
+      <c r="B220" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C220" s="5"/>
-      <c r="D220" s="3"/>
-      <c r="E220" s="43"/>
-      <c r="F220" s="7"/>
+      <c r="D220" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E220" s="43">
+        <v>2600</v>
+      </c>
+      <c r="F220" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="221" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B221" s="11"/>
+      <c r="B221" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C221" s="5"/>
-      <c r="D221" s="3"/>
-      <c r="E221" s="43"/>
-      <c r="F221" s="7"/>
+      <c r="D221" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E221" s="43">
+        <v>1440</v>
+      </c>
+      <c r="F221" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="222" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B222" s="11"/>
+      <c r="B222" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C222" s="5"/>
-      <c r="D222" s="3"/>
-      <c r="E222" s="43"/>
-      <c r="F222" s="7"/>
+      <c r="D222" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E222" s="43">
+        <v>89.84</v>
+      </c>
+      <c r="F222" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="223" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B223" s="11"/>
+      <c r="B223" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C223" s="5"/>
-      <c r="D223" s="3"/>
-      <c r="E223" s="43"/>
-      <c r="F223" s="7"/>
+      <c r="D223" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E223" s="43">
+        <v>635</v>
+      </c>
+      <c r="F223" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="224" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B224" s="11"/>
+      <c r="B224" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C224" s="5"/>
-      <c r="D224" s="3"/>
-      <c r="E224" s="43"/>
-      <c r="F224" s="7"/>
+      <c r="D224" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E224" s="43">
+        <v>44</v>
+      </c>
+      <c r="F224" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="225" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B225" s="11"/>
+      <c r="B225" s="11" t="s">
+        <v>169</v>
+      </c>
       <c r="C225" s="5"/>
-      <c r="D225" s="3"/>
-      <c r="E225" s="43"/>
-      <c r="F225" s="7"/>
+      <c r="D225" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E225" s="43">
+        <v>55</v>
+      </c>
+      <c r="F225" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="226" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B226" s="11"/>
+      <c r="B226" s="11" t="s">
+        <v>112</v>
+      </c>
       <c r="C226" s="5"/>
-      <c r="D226" s="3"/>
-      <c r="E226" s="43"/>
-      <c r="F226" s="7"/>
+      <c r="D226" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E226" s="43">
+        <v>120</v>
+      </c>
+      <c r="F226" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="227" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B227" s="11"/>
+      <c r="B227" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C227" s="5"/>
-      <c r="D227" s="3"/>
-      <c r="E227" s="43"/>
-      <c r="F227" s="7"/>
+      <c r="D227" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E227" s="43">
+        <v>200</v>
+      </c>
+      <c r="F227" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="228" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B228" s="11"/>
+      <c r="B228" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C228" s="5"/>
-      <c r="D228" s="3"/>
-      <c r="E228" s="43"/>
-      <c r="F228" s="7"/>
+      <c r="D228" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E228" s="43">
+        <v>175</v>
+      </c>
+      <c r="F228" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="229" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B229" s="11"/>
+      <c r="B229" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C229" s="5"/>
-      <c r="D229" s="3"/>
-      <c r="E229" s="43"/>
-      <c r="F229" s="7"/>
+      <c r="D229" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E229" s="43">
+        <v>205</v>
+      </c>
+      <c r="F229" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="230" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B230" s="11"/>
+      <c r="B230" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C230" s="5"/>
-      <c r="D230" s="3"/>
-      <c r="E230" s="43"/>
-      <c r="F230" s="7"/>
+      <c r="D230" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E230" s="43">
+        <v>200</v>
+      </c>
+      <c r="F230" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="231" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B231" s="11"/>
+      <c r="B231" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C231" s="5"/>
-      <c r="D231" s="3"/>
-      <c r="E231" s="43"/>
-      <c r="F231" s="7"/>
+      <c r="D231" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E231" s="43">
+        <v>3500</v>
+      </c>
+      <c r="F231" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="232" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B232" s="11"/>
+      <c r="B232" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C232" s="5"/>
-      <c r="D232" s="3"/>
-      <c r="E232" s="43"/>
-      <c r="F232" s="7"/>
+      <c r="D232" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E232" s="43">
+        <v>60</v>
+      </c>
+      <c r="F232" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="233" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B233" s="11"/>
+      <c r="B233" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C233" s="5"/>
-      <c r="D233" s="3"/>
-      <c r="E233" s="43"/>
-      <c r="F233" s="7"/>
+      <c r="D233" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E233" s="43">
+        <v>219</v>
+      </c>
+      <c r="F233" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="234" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B234" s="11"/>
+      <c r="B234" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C234" s="5"/>
-      <c r="D234" s="3"/>
-      <c r="E234" s="43"/>
-      <c r="F234" s="7"/>
+      <c r="D234" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E234" s="43">
+        <v>105</v>
+      </c>
+      <c r="F234" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="235" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B235" s="11"/>
+      <c r="B235" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C235" s="5"/>
-      <c r="D235" s="3"/>
-      <c r="E235" s="43"/>
-      <c r="F235" s="7"/>
+      <c r="D235" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E235" s="43">
+        <v>1950</v>
+      </c>
+      <c r="F235" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="236" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B236" s="11"/>
+      <c r="B236" s="11" t="s">
+        <v>167</v>
+      </c>
       <c r="C236" s="5"/>
-      <c r="D236" s="3"/>
-      <c r="E236" s="43"/>
-      <c r="F236" s="7"/>
+      <c r="D236" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E236" s="43">
+        <v>70</v>
+      </c>
+      <c r="F236" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="237" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B237" s="11"/>
+      <c r="B237" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C237" s="5"/>
-      <c r="D237" s="3"/>
-      <c r="E237" s="43"/>
-      <c r="F237" s="7"/>
+      <c r="D237" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E237" s="43">
+        <v>70</v>
+      </c>
+      <c r="F237" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="238" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B238" s="11"/>
+      <c r="B238" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C238" s="5"/>
-      <c r="D238" s="3"/>
-      <c r="E238" s="43"/>
-      <c r="F238" s="7"/>
+      <c r="D238" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E238" s="43">
+        <v>35</v>
+      </c>
+      <c r="F238" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="239" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B239" s="11"/>
+      <c r="B239" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C239" s="5"/>
-      <c r="D239" s="3"/>
-      <c r="E239" s="43"/>
-      <c r="F239" s="7"/>
+      <c r="D239" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E239" s="43">
+        <v>7320</v>
+      </c>
+      <c r="F239" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="240" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B240" s="11"/>
+      <c r="B240" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C240" s="5"/>
-      <c r="D240" s="3"/>
-      <c r="E240" s="43"/>
-      <c r="F240" s="7"/>
+      <c r="D240" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E240" s="43">
+        <v>346</v>
+      </c>
+      <c r="F240" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="241" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B241" s="11"/>
+      <c r="B241" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C241" s="5"/>
-      <c r="D241" s="3"/>
-      <c r="E241" s="43"/>
-      <c r="F241" s="7"/>
+      <c r="D241" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E241" s="43">
+        <v>50</v>
+      </c>
+      <c r="F241" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="242" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B242" s="11"/>
+      <c r="B242" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C242" s="5"/>
-      <c r="D242" s="3"/>
-      <c r="E242" s="43"/>
-      <c r="F242" s="7"/>
+      <c r="D242" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E242" s="43">
+        <v>100</v>
+      </c>
+      <c r="F242" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="243" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B243" s="11"/>
+      <c r="B243" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C243" s="5"/>
-      <c r="D243" s="3"/>
-      <c r="E243" s="43"/>
-      <c r="F243" s="7"/>
+      <c r="D243" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E243" s="43">
+        <v>394.38</v>
+      </c>
+      <c r="F243" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="244" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B244" s="11"/>
+      <c r="B244" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C244" s="5"/>
-      <c r="D244" s="3"/>
-      <c r="E244" s="43"/>
-      <c r="F244" s="7"/>
+      <c r="D244" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="E244" s="43">
+        <v>78</v>
+      </c>
+      <c r="F244" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="245" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B245" s="11"/>
+      <c r="B245" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C245" s="5"/>
-      <c r="D245" s="3"/>
-      <c r="E245" s="43"/>
-      <c r="F245" s="7"/>
+      <c r="D245" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E245" s="43">
+        <v>190</v>
+      </c>
+      <c r="F245" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="246" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B246" s="11"/>
+      <c r="B246" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C246" s="5"/>
-      <c r="D246" s="3"/>
-      <c r="E246" s="43"/>
-      <c r="F246" s="7"/>
+      <c r="D246" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E246" s="43">
+        <v>50</v>
+      </c>
+      <c r="F246" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="247" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B247" s="11"/>
+      <c r="B247" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C247" s="5"/>
-      <c r="D247" s="3"/>
-      <c r="E247" s="43"/>
-      <c r="F247" s="7"/>
+      <c r="D247" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E247" s="43">
+        <v>630</v>
+      </c>
+      <c r="F247" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="248" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B248" s="11"/>
+      <c r="B248" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C248" s="5"/>
-      <c r="D248" s="3"/>
-      <c r="E248" s="43"/>
-      <c r="F248" s="7"/>
+      <c r="D248" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E248" s="43">
+        <v>2778</v>
+      </c>
+      <c r="F248" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="249" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B249" s="11"/>
+      <c r="B249" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C249" s="5"/>
-      <c r="D249" s="3"/>
-      <c r="E249" s="43"/>
-      <c r="F249" s="7"/>
+      <c r="D249" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E249" s="43">
+        <v>592</v>
+      </c>
+      <c r="F249" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="250" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B250" s="11"/>
+      <c r="B250" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C250" s="5"/>
-      <c r="D250" s="3"/>
-      <c r="E250" s="43"/>
-      <c r="F250" s="7"/>
+      <c r="D250" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E250" s="43">
+        <v>1012.35</v>
+      </c>
+      <c r="F250" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="251" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B251" s="11"/>
+      <c r="B251" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C251" s="5"/>
-      <c r="D251" s="3"/>
-      <c r="E251" s="43"/>
-      <c r="F251" s="7"/>
+      <c r="D251" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E251" s="43">
+        <v>580</v>
+      </c>
+      <c r="F251" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="252" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B252" s="11"/>
+      <c r="B252" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C252" s="5"/>
-      <c r="D252" s="3"/>
-      <c r="E252" s="43"/>
-      <c r="F252" s="7"/>
+      <c r="D252" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E252" s="43">
+        <v>185</v>
+      </c>
+      <c r="F252" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="253" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B253" s="11"/>
+      <c r="B253" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C253" s="5"/>
-      <c r="D253" s="3"/>
-      <c r="E253" s="43"/>
-      <c r="F253" s="7"/>
+      <c r="D253" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E253" s="43">
+        <v>60</v>
+      </c>
+      <c r="F253" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="254" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B254" s="11"/>
+      <c r="B254" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C254" s="5"/>
-      <c r="D254" s="3"/>
-      <c r="E254" s="43"/>
-      <c r="F254" s="7"/>
+      <c r="D254" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E254" s="43">
+        <v>12156</v>
+      </c>
+      <c r="F254" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="255" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B255" s="11"/>
+      <c r="B255" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C255" s="5"/>
-      <c r="D255" s="3"/>
-      <c r="E255" s="43"/>
-      <c r="F255" s="7"/>
+      <c r="D255" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E255" s="43">
+        <v>16800</v>
+      </c>
+      <c r="F255" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="256" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B256" s="11"/>
+      <c r="B256" s="11" t="s">
+        <v>167</v>
+      </c>
       <c r="C256" s="5"/>
-      <c r="D256" s="3"/>
-      <c r="E256" s="43"/>
-      <c r="F256" s="7"/>
+      <c r="D256" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E256" s="43">
+        <v>97</v>
+      </c>
+      <c r="F256" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="257" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B257" s="11"/>
+      <c r="B257" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C257" s="5"/>
-      <c r="D257" s="3"/>
-      <c r="E257" s="43"/>
-      <c r="F257" s="7"/>
+      <c r="D257" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E257" s="43">
+        <v>1392</v>
+      </c>
+      <c r="F257" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="258" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B258" s="11"/>
+      <c r="B258" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C258" s="5"/>
-      <c r="D258" s="3"/>
-      <c r="E258" s="43"/>
-      <c r="F258" s="7"/>
+      <c r="D258" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E258" s="43">
+        <v>1245</v>
+      </c>
+      <c r="F258" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="259" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B259" s="11"/>
+      <c r="B259" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C259" s="5"/>
-      <c r="D259" s="3"/>
-      <c r="E259" s="43"/>
-      <c r="F259" s="7"/>
+      <c r="D259" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E259" s="43">
+        <v>712</v>
+      </c>
+      <c r="F259" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="260" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B260" s="11"/>
+      <c r="B260" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C260" s="5"/>
-      <c r="D260" s="3"/>
-      <c r="E260" s="43"/>
-      <c r="F260" s="7"/>
+      <c r="D260" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E260" s="43">
+        <v>1420</v>
+      </c>
+      <c r="F260" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="261" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B261" s="11"/>
+      <c r="B261" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C261" s="5"/>
-      <c r="D261" s="3"/>
-      <c r="E261" s="43"/>
-      <c r="F261" s="7"/>
+      <c r="D261" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E261" s="43">
+        <v>696</v>
+      </c>
+      <c r="F261" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="262" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B262" s="11"/>
+      <c r="B262" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C262" s="5"/>
-      <c r="D262" s="3"/>
-      <c r="E262" s="43"/>
-      <c r="F262" s="7"/>
+      <c r="D262" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E262" s="43">
+        <v>100</v>
+      </c>
+      <c r="F262" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="263" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B263" s="11"/>
+      <c r="B263" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C263" s="5"/>
-      <c r="D263" s="3"/>
-      <c r="E263" s="43"/>
-      <c r="F263" s="7"/>
+      <c r="D263" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E263" s="43">
+        <v>40</v>
+      </c>
+      <c r="F263" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="264" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B264" s="11"/>
+      <c r="B264" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C264" s="5"/>
-      <c r="D264" s="3"/>
-      <c r="E264" s="43"/>
-      <c r="F264" s="7"/>
+      <c r="D264" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E264" s="43">
+        <v>108</v>
+      </c>
+      <c r="F264" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="265" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B265" s="11"/>
+      <c r="B265" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C265" s="5"/>
-      <c r="D265" s="3"/>
-      <c r="E265" s="43"/>
-      <c r="F265" s="7"/>
+      <c r="D265" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E265" s="43">
+        <v>66</v>
+      </c>
+      <c r="F265" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="266" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B266" s="11"/>
+      <c r="B266" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C266" s="5"/>
-      <c r="D266" s="3"/>
-      <c r="E266" s="43"/>
-      <c r="F266" s="7"/>
+      <c r="D266" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E266" s="43">
+        <v>200</v>
+      </c>
+      <c r="F266" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="267" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B267" s="11"/>
+      <c r="B267" s="11" t="s">
+        <v>12</v>
+      </c>
       <c r="C267" s="5"/>
-      <c r="D267" s="3"/>
-      <c r="E267" s="43"/>
-      <c r="F267" s="7"/>
+      <c r="D267" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="E267" s="43">
+        <v>1200</v>
+      </c>
+      <c r="F267" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="268" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B268" s="11"/>
+      <c r="B268" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C268" s="5"/>
-      <c r="D268" s="3"/>
-      <c r="E268" s="43"/>
-      <c r="F268" s="7"/>
+      <c r="D268" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E268" s="43">
+        <v>10</v>
+      </c>
+      <c r="F268" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="269" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B269" s="11"/>
+      <c r="B269" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C269" s="5"/>
-      <c r="D269" s="3"/>
-      <c r="E269" s="43"/>
-      <c r="F269" s="7"/>
+      <c r="D269" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E269" s="43">
+        <v>180</v>
+      </c>
+      <c r="F269" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="270" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B270" s="11"/>
+      <c r="B270" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C270" s="5"/>
-      <c r="D270" s="3"/>
-      <c r="E270" s="43"/>
-      <c r="F270" s="7"/>
+      <c r="D270" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E270" s="43">
+        <v>280</v>
+      </c>
+      <c r="F270" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="271" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B271" s="11"/>
+      <c r="B271" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C271" s="5"/>
-      <c r="D271" s="3"/>
-      <c r="E271" s="43"/>
-      <c r="F271" s="7"/>
+      <c r="D271" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E271" s="43">
+        <v>210</v>
+      </c>
+      <c r="F271" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="272" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B272" s="11"/>
+      <c r="B272" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C272" s="5"/>
-      <c r="D272" s="3"/>
-      <c r="E272" s="43"/>
-      <c r="F272" s="7"/>
+      <c r="D272" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E272" s="43">
+        <v>250</v>
+      </c>
+      <c r="F272" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="273" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B273" s="11"/>
+      <c r="B273" s="11" t="s">
+        <v>167</v>
+      </c>
       <c r="C273" s="5"/>
-      <c r="D273" s="3"/>
-      <c r="E273" s="43"/>
-      <c r="F273" s="7"/>
+      <c r="D273" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E273" s="43">
+        <v>309.72000000000003</v>
+      </c>
+      <c r="F273" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="274" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B274" s="11"/>
+      <c r="B274" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C274" s="5"/>
-      <c r="D274" s="3"/>
-      <c r="E274" s="43"/>
-      <c r="F274" s="7"/>
+      <c r="D274" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E274" s="43">
+        <v>265.60000000000002</v>
+      </c>
+      <c r="F274" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="275" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B275" s="11"/>
+      <c r="B275" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C275" s="5"/>
-      <c r="D275" s="3"/>
-      <c r="E275" s="43"/>
-      <c r="F275" s="7"/>
+      <c r="D275" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E275" s="43">
+        <v>263</v>
+      </c>
+      <c r="F275" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="276" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B276" s="11"/>
+      <c r="B276" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C276" s="5"/>
-      <c r="D276" s="3"/>
-      <c r="E276" s="43"/>
-      <c r="F276" s="7"/>
+      <c r="D276" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E276" s="43">
+        <v>150</v>
+      </c>
+      <c r="F276" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="277" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B277" s="11"/>
+      <c r="B277" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C277" s="5"/>
-      <c r="D277" s="3"/>
-      <c r="E277" s="43"/>
-      <c r="F277" s="7"/>
+      <c r="D277" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E277" s="43">
+        <v>100</v>
+      </c>
+      <c r="F277" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="278" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B278" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-18 15:56
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="363" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6340FEDA-37CA-457D-B2E0-A5895F5A1E2A}"/>
+  <xr:revisionPtr revIDLastSave="386" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{461B6FF1-0012-4F9F-9BCA-A49BBC422EC9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2718" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2729" uniqueCount="172">
   <si>
     <t>Custo</t>
   </si>
@@ -43773,46 +43773,92 @@
       </c>
     </row>
     <row r="278" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B278" s="11"/>
+      <c r="B278" s="11" t="s">
+        <v>31</v>
+      </c>
       <c r="C278" s="5"/>
-      <c r="D278" s="3"/>
-      <c r="E278" s="43"/>
-      <c r="F278" s="7"/>
+      <c r="D278" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E278" s="43">
+        <v>33</v>
+      </c>
+      <c r="F278" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="279" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B279" s="11"/>
+      <c r="B279" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C279" s="5"/>
       <c r="D279" s="3"/>
-      <c r="E279" s="43"/>
-      <c r="F279" s="7"/>
+      <c r="E279" s="43">
+        <v>410</v>
+      </c>
+      <c r="F279" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="280" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B280" s="11"/>
+      <c r="B280" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C280" s="5"/>
-      <c r="D280" s="3"/>
-      <c r="E280" s="43"/>
-      <c r="F280" s="7"/>
+      <c r="D280" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E280" s="43">
+        <v>450</v>
+      </c>
+      <c r="F280" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="281" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B281" s="11"/>
+      <c r="B281" s="11" t="s">
+        <v>142</v>
+      </c>
       <c r="C281" s="5"/>
-      <c r="D281" s="3"/>
-      <c r="E281" s="43"/>
-      <c r="F281" s="7"/>
+      <c r="D281" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E281" s="43">
+        <v>50</v>
+      </c>
+      <c r="F281" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="282" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B282" s="11"/>
+      <c r="B282" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C282" s="5"/>
-      <c r="D282" s="3"/>
-      <c r="E282" s="43"/>
-      <c r="F282" s="7"/>
+      <c r="D282" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E282" s="43">
+        <v>150</v>
+      </c>
+      <c r="F282" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="283" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B283" s="11"/>
+      <c r="B283" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C283" s="5"/>
-      <c r="D283" s="3"/>
-      <c r="E283" s="43"/>
-      <c r="F283" s="7"/>
+      <c r="D283" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E283" s="43">
+        <v>690</v>
+      </c>
+      <c r="F283" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="284" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B284" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-03-30 11:39
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="386" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{461B6FF1-0012-4F9F-9BCA-A49BBC422EC9}"/>
+  <xr:revisionPtr revIDLastSave="528" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFE480CF-7CE6-44C1-B2EE-93EAF9F9936A}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2729" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2795" uniqueCount="175">
   <si>
     <t>Custo</t>
   </si>
@@ -557,6 +557,15 @@
   </si>
   <si>
     <t>MANG DIVI</t>
+  </si>
+  <si>
+    <t>GW LANTERNAGEM</t>
+  </si>
+  <si>
+    <t>GBAPNEUS</t>
+  </si>
+  <si>
+    <t>NORTE FREIOS</t>
   </si>
 </sst>
 </file>
@@ -43861,235 +43870,499 @@
       </c>
     </row>
     <row r="284" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B284" s="11"/>
+      <c r="B284" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="C284" s="5"/>
-      <c r="D284" s="3"/>
-      <c r="E284" s="43"/>
-      <c r="F284" s="7"/>
+      <c r="D284" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="E284" s="43">
+        <v>7000</v>
+      </c>
+      <c r="F284" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="285" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B285" s="11"/>
+      <c r="B285" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C285" s="5"/>
-      <c r="D285" s="3"/>
-      <c r="E285" s="43"/>
-      <c r="F285" s="7"/>
+      <c r="D285" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E285" s="43">
+        <v>190</v>
+      </c>
+      <c r="F285" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="286" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B286" s="11"/>
+      <c r="B286" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C286" s="5"/>
-      <c r="D286" s="3"/>
-      <c r="E286" s="43"/>
-      <c r="F286" s="7"/>
+      <c r="D286" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E286" s="43">
+        <v>193</v>
+      </c>
+      <c r="F286" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="287" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B287" s="11"/>
+      <c r="B287" s="11" t="s">
+        <v>142</v>
+      </c>
       <c r="C287" s="5"/>
-      <c r="D287" s="3"/>
-      <c r="E287" s="43"/>
-      <c r="F287" s="7"/>
+      <c r="D287" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E287" s="43">
+        <v>80</v>
+      </c>
+      <c r="F287" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="288" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B288" s="11"/>
+      <c r="B288" s="11" t="s">
+        <v>142</v>
+      </c>
       <c r="C288" s="5"/>
-      <c r="D288" s="3"/>
-      <c r="E288" s="43"/>
-      <c r="F288" s="7"/>
+      <c r="D288" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E288" s="43">
+        <v>432</v>
+      </c>
+      <c r="F288" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="289" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B289" s="11"/>
+      <c r="B289" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C289" s="5"/>
-      <c r="D289" s="3"/>
-      <c r="E289" s="43"/>
-      <c r="F289" s="7"/>
+      <c r="D289" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E289" s="43">
+        <v>833.5</v>
+      </c>
+      <c r="F289" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="290" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B290" s="11"/>
+      <c r="B290" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="C290" s="5"/>
-      <c r="D290" s="3"/>
-      <c r="E290" s="43"/>
-      <c r="F290" s="7"/>
+      <c r="D290" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E290" s="43">
+        <v>269</v>
+      </c>
+      <c r="F290" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="291" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B291" s="11"/>
+      <c r="B291" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C291" s="5"/>
-      <c r="D291" s="3"/>
-      <c r="E291" s="43"/>
-      <c r="F291" s="7"/>
+      <c r="D291" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E291" s="43">
+        <v>2861</v>
+      </c>
+      <c r="F291" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="292" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B292" s="11"/>
+      <c r="B292" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C292" s="5"/>
-      <c r="D292" s="3"/>
-      <c r="E292" s="43"/>
-      <c r="F292" s="7"/>
+      <c r="D292" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E292" s="43">
+        <v>100</v>
+      </c>
+      <c r="F292" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="293" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B293" s="11"/>
+      <c r="B293" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C293" s="5"/>
-      <c r="D293" s="3"/>
-      <c r="E293" s="43"/>
-      <c r="F293" s="7"/>
+      <c r="D293" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E293" s="43">
+        <v>40</v>
+      </c>
+      <c r="F293" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="294" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B294" s="11"/>
+      <c r="B294" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C294" s="5"/>
-      <c r="D294" s="3"/>
-      <c r="E294" s="43"/>
-      <c r="F294" s="7"/>
+      <c r="D294" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E294" s="43">
+        <v>60</v>
+      </c>
+      <c r="F294" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="295" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B295" s="11"/>
+      <c r="B295" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C295" s="5"/>
-      <c r="D295" s="3"/>
-      <c r="E295" s="43"/>
-      <c r="F295" s="7"/>
+      <c r="D295" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E295" s="43">
+        <v>251.1</v>
+      </c>
+      <c r="F295" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="296" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B296" s="11"/>
+      <c r="B296" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C296" s="5"/>
-      <c r="D296" s="3"/>
-      <c r="E296" s="43"/>
-      <c r="F296" s="7"/>
+      <c r="D296" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E296" s="43">
+        <v>600</v>
+      </c>
+      <c r="F296" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="297" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B297" s="11"/>
+      <c r="B297" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C297" s="5"/>
-      <c r="D297" s="3"/>
-      <c r="E297" s="43"/>
-      <c r="F297" s="7"/>
+      <c r="D297" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E297" s="43">
+        <v>902.1</v>
+      </c>
+      <c r="F297" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="298" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B298" s="11"/>
+      <c r="B298" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C298" s="5"/>
-      <c r="D298" s="3"/>
-      <c r="E298" s="43"/>
-      <c r="F298" s="7"/>
+      <c r="D298" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E298" s="43">
+        <v>200</v>
+      </c>
+      <c r="F298" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="299" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B299" s="11"/>
+      <c r="B299" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C299" s="5"/>
-      <c r="D299" s="3"/>
-      <c r="E299" s="43"/>
-      <c r="F299" s="7"/>
+      <c r="D299" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E299" s="43">
+        <v>50</v>
+      </c>
+      <c r="F299" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="300" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B300" s="11"/>
+      <c r="B300" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C300" s="5"/>
-      <c r="D300" s="3"/>
-      <c r="E300" s="43"/>
-      <c r="F300" s="7"/>
+      <c r="D300" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="E300" s="43">
+        <v>65</v>
+      </c>
+      <c r="F300" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="301" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B301" s="11"/>
+      <c r="B301" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C301" s="5"/>
-      <c r="D301" s="3"/>
-      <c r="E301" s="43"/>
-      <c r="F301" s="7"/>
+      <c r="D301" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E301" s="43">
+        <v>200</v>
+      </c>
+      <c r="F301" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="302" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B302" s="11"/>
+      <c r="B302" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C302" s="5"/>
-      <c r="D302" s="3"/>
-      <c r="E302" s="43"/>
-      <c r="F302" s="7"/>
+      <c r="D302" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E302" s="43">
+        <v>185</v>
+      </c>
+      <c r="F302" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="303" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B303" s="11"/>
+      <c r="B303" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C303" s="5"/>
-      <c r="D303" s="3"/>
-      <c r="E303" s="43"/>
-      <c r="F303" s="7"/>
+      <c r="D303" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E303" s="43">
+        <v>128.25</v>
+      </c>
+      <c r="F303" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="304" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B304" s="11"/>
+      <c r="B304" s="11" t="s">
+        <v>142</v>
+      </c>
       <c r="C304" s="5"/>
-      <c r="D304" s="3"/>
-      <c r="E304" s="43"/>
-      <c r="F304" s="7"/>
+      <c r="D304" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E304" s="43">
+        <v>410.5</v>
+      </c>
+      <c r="F304" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="305" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B305" s="11"/>
+      <c r="B305" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C305" s="5"/>
-      <c r="D305" s="3"/>
-      <c r="E305" s="43"/>
-      <c r="F305" s="7"/>
+      <c r="D305" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E305" s="43">
+        <v>1113.3</v>
+      </c>
+      <c r="F305" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="306" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B306" s="11"/>
+      <c r="B306" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C306" s="5"/>
-      <c r="D306" s="3"/>
-      <c r="E306" s="43"/>
-      <c r="F306" s="7"/>
+      <c r="D306" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E306" s="43">
+        <v>350</v>
+      </c>
+      <c r="F306" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="307" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B307" s="11"/>
+      <c r="B307" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C307" s="5"/>
-      <c r="D307" s="3"/>
-      <c r="E307" s="43"/>
-      <c r="F307" s="7"/>
+      <c r="D307" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E307" s="43">
+        <v>1509.86</v>
+      </c>
+      <c r="F307" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="308" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B308" s="11"/>
+      <c r="B308" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C308" s="5"/>
-      <c r="D308" s="3"/>
-      <c r="E308" s="43"/>
-      <c r="F308" s="7"/>
+      <c r="D308" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E308" s="43">
+        <v>2110</v>
+      </c>
+      <c r="F308" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="309" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B309" s="11"/>
+      <c r="B309" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C309" s="5"/>
-      <c r="D309" s="3"/>
-      <c r="E309" s="43"/>
-      <c r="F309" s="7"/>
+      <c r="D309" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E309" s="43">
+        <v>802</v>
+      </c>
+      <c r="F309" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="310" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B310" s="11"/>
+      <c r="B310" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C310" s="5"/>
-      <c r="D310" s="3"/>
-      <c r="E310" s="43"/>
-      <c r="F310" s="7"/>
+      <c r="D310" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E310" s="43">
+        <v>200</v>
+      </c>
+      <c r="F310" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="311" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B311" s="11"/>
+      <c r="B311" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C311" s="5"/>
-      <c r="D311" s="3"/>
-      <c r="E311" s="43"/>
-      <c r="F311" s="7"/>
+      <c r="D311" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E311" s="43">
+        <v>934</v>
+      </c>
+      <c r="F311" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="312" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B312" s="11"/>
+      <c r="B312" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C312" s="5"/>
-      <c r="D312" s="3"/>
-      <c r="E312" s="43"/>
-      <c r="F312" s="7"/>
+      <c r="D312" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E312" s="43">
+        <v>1460</v>
+      </c>
+      <c r="F312" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="313" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B313" s="11"/>
+      <c r="B313" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C313" s="5"/>
-      <c r="D313" s="3"/>
-      <c r="E313" s="43"/>
-      <c r="F313" s="7"/>
+      <c r="D313" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E313" s="43">
+        <v>3250</v>
+      </c>
+      <c r="F313" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="314" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B314" s="11"/>
+      <c r="B314" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C314" s="5"/>
-      <c r="D314" s="3"/>
-      <c r="E314" s="43"/>
-      <c r="F314" s="7"/>
+      <c r="D314" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E314" s="43">
+        <v>100</v>
+      </c>
+      <c r="F314" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="315" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B315" s="11"/>
+      <c r="B315" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C315" s="5"/>
-      <c r="D315" s="3"/>
-      <c r="E315" s="43"/>
-      <c r="F315" s="7"/>
+      <c r="D315" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E315" s="43">
+        <v>250</v>
+      </c>
+      <c r="F315" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="316" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B316" s="11"/>
+      <c r="B316" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C316" s="5"/>
-      <c r="D316" s="3"/>
-      <c r="E316" s="43"/>
-      <c r="F316" s="7"/>
+      <c r="D316" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E316" s="43">
+        <v>2096</v>
+      </c>
+      <c r="F316" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="317" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B317" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-04-01 16:54
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="528" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFE480CF-7CE6-44C1-B2EE-93EAF9F9936A}"/>
+  <xr:revisionPtr revIDLastSave="581" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFDF2FBC-8492-4091-98B2-99EDC29E3E6A}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
+    <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2795" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2821" uniqueCount="175">
   <si>
     <t>Custo</t>
   </si>
@@ -44365,95 +44365,199 @@
       </c>
     </row>
     <row r="317" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B317" s="11"/>
+      <c r="B317" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C317" s="5"/>
-      <c r="D317" s="3"/>
-      <c r="E317" s="43"/>
-      <c r="F317" s="7"/>
+      <c r="D317" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E317" s="43">
+        <v>671</v>
+      </c>
+      <c r="F317" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="318" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B318" s="11"/>
+      <c r="B318" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C318" s="5"/>
-      <c r="D318" s="3"/>
-      <c r="E318" s="43"/>
-      <c r="F318" s="7"/>
+      <c r="D318" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E318" s="43">
+        <v>530</v>
+      </c>
+      <c r="F318" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="319" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B319" s="11"/>
+      <c r="B319" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C319" s="5"/>
-      <c r="D319" s="3"/>
-      <c r="E319" s="43"/>
-      <c r="F319" s="7"/>
+      <c r="D319" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E319" s="43">
+        <v>70</v>
+      </c>
+      <c r="F319" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="320" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B320" s="11"/>
+      <c r="B320" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C320" s="5"/>
-      <c r="D320" s="3"/>
-      <c r="E320" s="43"/>
-      <c r="F320" s="7"/>
+      <c r="D320" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E320" s="43">
+        <v>200</v>
+      </c>
+      <c r="F320" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="321" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B321" s="11"/>
+      <c r="B321" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="C321" s="5"/>
-      <c r="D321" s="3"/>
-      <c r="E321" s="43"/>
-      <c r="F321" s="7"/>
+      <c r="D321" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E321" s="43">
+        <v>1101</v>
+      </c>
+      <c r="F321" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="322" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B322" s="11"/>
+      <c r="B322" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C322" s="5"/>
-      <c r="D322" s="3"/>
-      <c r="E322" s="43"/>
-      <c r="F322" s="7"/>
+      <c r="D322" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="E322" s="43">
+        <v>213.6</v>
+      </c>
+      <c r="F322" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="323" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B323" s="11"/>
+      <c r="B323" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C323" s="5"/>
-      <c r="D323" s="3"/>
-      <c r="E323" s="43"/>
-      <c r="F323" s="7"/>
+      <c r="D323" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E323" s="43">
+        <v>280</v>
+      </c>
+      <c r="F323" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="324" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B324" s="11"/>
+      <c r="B324" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C324" s="5"/>
-      <c r="D324" s="3"/>
-      <c r="E324" s="43"/>
-      <c r="F324" s="7"/>
+      <c r="D324" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E324" s="43">
+        <v>345</v>
+      </c>
+      <c r="F324" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="325" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B325" s="11"/>
+      <c r="B325" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C325" s="5"/>
-      <c r="D325" s="3"/>
-      <c r="E325" s="43"/>
-      <c r="F325" s="7"/>
+      <c r="D325" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E325" s="43">
+        <v>288</v>
+      </c>
+      <c r="F325" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="326" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B326" s="11"/>
+      <c r="B326" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C326" s="5"/>
-      <c r="D326" s="3"/>
-      <c r="E326" s="43"/>
-      <c r="F326" s="7"/>
+      <c r="D326" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E326" s="43">
+        <v>1335</v>
+      </c>
+      <c r="F326" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="327" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B327" s="11"/>
+      <c r="B327" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C327" s="5"/>
-      <c r="D327" s="3"/>
-      <c r="E327" s="43"/>
-      <c r="F327" s="7"/>
+      <c r="D327" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E327" s="43">
+        <v>3500</v>
+      </c>
+      <c r="F327" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="328" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B328" s="11"/>
+      <c r="B328" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C328" s="5"/>
-      <c r="D328" s="3"/>
-      <c r="E328" s="43"/>
-      <c r="F328" s="7"/>
+      <c r="D328" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E328" s="43">
+        <v>175</v>
+      </c>
+      <c r="F328" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="329" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B329" s="11"/>
+      <c r="B329" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C329" s="5"/>
-      <c r="D329" s="3"/>
-      <c r="E329" s="43"/>
-      <c r="F329" s="7"/>
+      <c r="D329" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E329" s="43">
+        <v>960</v>
+      </c>
+      <c r="F329" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="330" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B330" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-04-02 17:25
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="581" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DFDF2FBC-8492-4091-98B2-99EDC29E3E6A}"/>
+  <xr:revisionPtr revIDLastSave="613" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{371E4FA9-A655-47FA-A8BF-0C060F3CEF65}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2821" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2837" uniqueCount="180">
   <si>
     <t>Custo</t>
   </si>
@@ -566,6 +566,21 @@
   </si>
   <si>
     <t>NORTE FREIOS</t>
+  </si>
+  <si>
+    <t>AUTO CENTRO TUDO CAR</t>
+  </si>
+  <si>
+    <t>AO ELETRICA DO LEO</t>
+  </si>
+  <si>
+    <t>BORRACHARIA  CARGA PESADA</t>
+  </si>
+  <si>
+    <t>BORRACHARIA DO DEVIS</t>
+  </si>
+  <si>
+    <t>HIDRAUMANG</t>
   </si>
 </sst>
 </file>
@@ -44560,60 +44575,124 @@
       </c>
     </row>
     <row r="330" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B330" s="11"/>
+      <c r="B330" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C330" s="5"/>
-      <c r="D330" s="3"/>
-      <c r="E330" s="43"/>
-      <c r="F330" s="7"/>
+      <c r="D330" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E330" s="43">
+        <v>50</v>
+      </c>
+      <c r="F330" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="331" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B331" s="11"/>
+      <c r="B331" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C331" s="5"/>
-      <c r="D331" s="3"/>
-      <c r="E331" s="43"/>
-      <c r="F331" s="7"/>
+      <c r="D331" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E331" s="43">
+        <v>200</v>
+      </c>
+      <c r="F331" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="332" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B332" s="11"/>
+      <c r="B332" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="C332" s="5"/>
-      <c r="D332" s="3"/>
-      <c r="E332" s="43"/>
-      <c r="F332" s="7"/>
+      <c r="D332" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="E332" s="43">
+        <v>200</v>
+      </c>
+      <c r="F332" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="333" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B333" s="11"/>
+      <c r="B333" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C333" s="5"/>
-      <c r="D333" s="3"/>
-      <c r="E333" s="43"/>
-      <c r="F333" s="7"/>
+      <c r="D333" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="E333" s="43">
+        <v>161.30000000000001</v>
+      </c>
+      <c r="F333" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="334" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B334" s="11"/>
+      <c r="B334" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C334" s="5"/>
-      <c r="D334" s="3"/>
-      <c r="E334" s="43"/>
-      <c r="F334" s="7"/>
+      <c r="D334" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="E334" s="43">
+        <v>110</v>
+      </c>
+      <c r="F334" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="335" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B335" s="11"/>
+      <c r="B335" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C335" s="5"/>
-      <c r="D335" s="3"/>
-      <c r="E335" s="43"/>
-      <c r="F335" s="7"/>
+      <c r="D335" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E335" s="43">
+        <v>192.2</v>
+      </c>
+      <c r="F335" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="336" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B336" s="11"/>
+      <c r="B336" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C336" s="5"/>
-      <c r="D336" s="3"/>
-      <c r="E336" s="43"/>
-      <c r="F336" s="7"/>
+      <c r="D336" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="E336" s="43">
+        <v>80</v>
+      </c>
+      <c r="F336" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="337" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B337" s="11"/>
+      <c r="B337" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C337" s="5"/>
-      <c r="D337" s="3"/>
-      <c r="E337" s="43"/>
-      <c r="F337" s="7"/>
+      <c r="D337" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="E337" s="43">
+        <v>30</v>
+      </c>
+      <c r="F337" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="338" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B338" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-05-06 17:15
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="613" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{371E4FA9-A655-47FA-A8BF-0C060F3CEF65}"/>
+  <xr:revisionPtr revIDLastSave="1109" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B71718C-E7FA-4FF4-8117-07FD318F6E2C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2837" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3078" uniqueCount="185">
   <si>
     <t>Custo</t>
   </si>
@@ -581,6 +581,21 @@
   </si>
   <si>
     <t>HIDRAUMANG</t>
+  </si>
+  <si>
+    <t>TEJ3A51</t>
+  </si>
+  <si>
+    <t>TOTAL PARTS ACESSORIOS</t>
+  </si>
+  <si>
+    <t>TDT2D85</t>
+  </si>
+  <si>
+    <t>ELI PNEUS</t>
+  </si>
+  <si>
+    <t>bombas injetoras</t>
   </si>
 </sst>
 </file>
@@ -44695,851 +44710,1817 @@
       </c>
     </row>
     <row r="338" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B338" s="11"/>
+      <c r="B338" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C338" s="5"/>
-      <c r="D338" s="3"/>
-      <c r="E338" s="43"/>
-      <c r="F338" s="7"/>
+      <c r="D338" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E338" s="43">
+        <v>1334</v>
+      </c>
+      <c r="F338" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="339" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B339" s="11"/>
+      <c r="B339" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C339" s="5"/>
-      <c r="D339" s="3"/>
-      <c r="E339" s="43"/>
-      <c r="F339" s="7"/>
+      <c r="D339" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E339" s="43">
+        <v>2967</v>
+      </c>
+      <c r="F339" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="340" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B340" s="11"/>
+      <c r="B340" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C340" s="5"/>
-      <c r="D340" s="3"/>
-      <c r="E340" s="43"/>
-      <c r="F340" s="7"/>
+      <c r="D340" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E340" s="43">
+        <v>110</v>
+      </c>
+      <c r="F340" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="341" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B341" s="11"/>
+      <c r="B341" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C341" s="5"/>
-      <c r="D341" s="3"/>
-      <c r="E341" s="43"/>
-      <c r="F341" s="7"/>
+      <c r="D341" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E341" s="43">
+        <v>160</v>
+      </c>
+      <c r="F341" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="342" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B342" s="11"/>
+      <c r="B342" s="11" t="s">
+        <v>39</v>
+      </c>
       <c r="C342" s="5"/>
-      <c r="D342" s="3"/>
-      <c r="E342" s="43"/>
-      <c r="F342" s="7"/>
+      <c r="D342" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E342" s="43">
+        <v>80</v>
+      </c>
+      <c r="F342" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="343" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B343" s="11"/>
+      <c r="B343" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C343" s="5"/>
-      <c r="D343" s="3"/>
-      <c r="E343" s="43"/>
-      <c r="F343" s="7"/>
+      <c r="D343" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E343" s="43">
+        <v>510</v>
+      </c>
+      <c r="F343" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="344" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B344" s="11"/>
+      <c r="B344" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C344" s="5"/>
-      <c r="D344" s="3"/>
-      <c r="E344" s="43"/>
-      <c r="F344" s="7"/>
+      <c r="D344" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E344" s="43">
+        <v>520</v>
+      </c>
+      <c r="F344" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="345" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B345" s="11"/>
+      <c r="B345" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C345" s="5"/>
-      <c r="D345" s="3"/>
-      <c r="E345" s="43"/>
-      <c r="F345" s="7"/>
+      <c r="D345" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E345" s="43">
+        <v>122.94</v>
+      </c>
+      <c r="F345" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="346" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B346" s="11"/>
+      <c r="B346" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C346" s="5"/>
-      <c r="D346" s="3"/>
-      <c r="E346" s="43"/>
-      <c r="F346" s="7"/>
+      <c r="D346" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E346" s="43">
+        <v>10002</v>
+      </c>
+      <c r="F346" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="347" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B347" s="11"/>
+      <c r="B347" s="11" t="s">
+        <v>180</v>
+      </c>
       <c r="C347" s="5"/>
       <c r="D347" s="3"/>
-      <c r="E347" s="43"/>
-      <c r="F347" s="7"/>
+      <c r="E347" s="43">
+        <v>90</v>
+      </c>
+      <c r="F347" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="348" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B348" s="11"/>
+      <c r="B348" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="C348" s="5"/>
-      <c r="D348" s="3"/>
-      <c r="E348" s="43"/>
-      <c r="F348" s="7"/>
+      <c r="D348" s="3" t="s">
+        <v>181</v>
+      </c>
+      <c r="E348" s="43">
+        <v>95</v>
+      </c>
+      <c r="F348" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="349" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B349" s="11"/>
+      <c r="B349" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C349" s="5"/>
-      <c r="D349" s="3"/>
-      <c r="E349" s="43"/>
-      <c r="F349" s="7"/>
+      <c r="D349" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E349" s="43">
+        <v>100</v>
+      </c>
+      <c r="F349" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="350" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B350" s="11"/>
+      <c r="B350" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C350" s="5"/>
-      <c r="D350" s="3"/>
-      <c r="E350" s="43"/>
-      <c r="F350" s="7"/>
+      <c r="D350" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E350" s="43">
+        <v>200</v>
+      </c>
+      <c r="F350" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="351" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B351" s="11"/>
+      <c r="B351" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C351" s="5"/>
-      <c r="D351" s="3"/>
-      <c r="E351" s="43"/>
-      <c r="F351" s="7"/>
+      <c r="D351" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E351" s="43">
+        <v>240</v>
+      </c>
+      <c r="F351" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="352" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B352" s="11"/>
+      <c r="B352" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C352" s="5"/>
-      <c r="D352" s="3"/>
-      <c r="E352" s="43"/>
-      <c r="F352" s="7"/>
+      <c r="D352" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E352" s="43">
+        <v>1010</v>
+      </c>
+      <c r="F352" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="353" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B353" s="11"/>
+      <c r="B353" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C353" s="5"/>
-      <c r="D353" s="3"/>
-      <c r="E353" s="43"/>
-      <c r="F353" s="7"/>
+      <c r="D353" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E353" s="43">
+        <v>556.6</v>
+      </c>
+      <c r="F353" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="354" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B354" s="11"/>
+      <c r="B354" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C354" s="5"/>
-      <c r="D354" s="3"/>
-      <c r="E354" s="43"/>
-      <c r="F354" s="7"/>
+      <c r="D354" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E354" s="43">
+        <v>185</v>
+      </c>
+      <c r="F354" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="355" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B355" s="11"/>
+      <c r="B355" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C355" s="5"/>
-      <c r="D355" s="3"/>
-      <c r="E355" s="43"/>
-      <c r="F355" s="7"/>
+      <c r="D355" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E355" s="43">
+        <v>140</v>
+      </c>
+      <c r="F355" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="356" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B356" s="11"/>
+      <c r="B356" s="11" t="s">
+        <v>182</v>
+      </c>
       <c r="C356" s="5"/>
-      <c r="D356" s="3"/>
-      <c r="E356" s="43"/>
-      <c r="F356" s="7"/>
+      <c r="D356" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E356" s="43">
+        <v>30</v>
+      </c>
+      <c r="F356" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="357" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B357" s="11"/>
+      <c r="B357" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C357" s="5"/>
-      <c r="D357" s="3"/>
-      <c r="E357" s="43"/>
-      <c r="F357" s="7"/>
+      <c r="D357" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E357" s="43">
+        <v>1020</v>
+      </c>
+      <c r="F357" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="358" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B358" s="11"/>
+      <c r="B358" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C358" s="5"/>
-      <c r="D358" s="3"/>
-      <c r="E358" s="43"/>
-      <c r="F358" s="7"/>
+      <c r="D358" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E358" s="43">
+        <v>1123</v>
+      </c>
+      <c r="F358" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="359" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B359" s="11"/>
+      <c r="B359" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C359" s="5"/>
-      <c r="D359" s="3"/>
-      <c r="E359" s="43"/>
-      <c r="F359" s="7"/>
+      <c r="D359" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E359" s="43">
+        <v>971</v>
+      </c>
+      <c r="F359" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="360" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B360" s="11"/>
+      <c r="B360" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C360" s="5"/>
-      <c r="D360" s="3"/>
-      <c r="E360" s="43"/>
-      <c r="F360" s="7"/>
+      <c r="D360" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E360" s="43">
+        <v>295</v>
+      </c>
+      <c r="F360" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="361" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B361" s="11"/>
+      <c r="B361" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C361" s="5"/>
-      <c r="D361" s="3"/>
-      <c r="E361" s="43"/>
-      <c r="F361" s="7"/>
+      <c r="D361" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E361" s="43">
+        <v>2858</v>
+      </c>
+      <c r="F361" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="362" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B362" s="11"/>
+      <c r="B362" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C362" s="5"/>
-      <c r="D362" s="3"/>
-      <c r="E362" s="43"/>
-      <c r="F362" s="7"/>
+      <c r="D362" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="E362" s="43">
+        <v>2150</v>
+      </c>
+      <c r="F362" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="363" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B363" s="11"/>
+      <c r="B363" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C363" s="5"/>
-      <c r="D363" s="3"/>
-      <c r="E363" s="43"/>
-      <c r="F363" s="7"/>
+      <c r="D363" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E363" s="43">
+        <v>100</v>
+      </c>
+      <c r="F363" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="364" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B364" s="11"/>
+      <c r="B364" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C364" s="5"/>
-      <c r="D364" s="3"/>
-      <c r="E364" s="43"/>
-      <c r="F364" s="7"/>
+      <c r="D364" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E364" s="43">
+        <v>370</v>
+      </c>
+      <c r="F364" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="365" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B365" s="11"/>
+      <c r="B365" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C365" s="5"/>
-      <c r="D365" s="3"/>
-      <c r="E365" s="43"/>
-      <c r="F365" s="7"/>
+      <c r="D365" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E365" s="43">
+        <v>1870</v>
+      </c>
+      <c r="F365" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="366" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B366" s="11"/>
+      <c r="B366" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C366" s="5"/>
-      <c r="D366" s="3"/>
-      <c r="E366" s="43"/>
-      <c r="F366" s="7"/>
+      <c r="D366" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E366" s="43">
+        <v>870</v>
+      </c>
+      <c r="F366" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="367" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B367" s="11"/>
+      <c r="B367" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C367" s="5"/>
-      <c r="D367" s="3"/>
-      <c r="E367" s="43"/>
-      <c r="F367" s="7"/>
+      <c r="D367" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E367" s="43">
+        <v>303</v>
+      </c>
+      <c r="F367" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="368" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B368" s="11"/>
+      <c r="B368" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C368" s="5"/>
-      <c r="D368" s="3"/>
-      <c r="E368" s="43"/>
-      <c r="F368" s="7"/>
+      <c r="D368" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="E368" s="43">
+        <v>250</v>
+      </c>
+      <c r="F368" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="369" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B369" s="11"/>
+      <c r="B369" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C369" s="5"/>
-      <c r="D369" s="3"/>
-      <c r="E369" s="43"/>
-      <c r="F369" s="7"/>
+      <c r="D369" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E369" s="43">
+        <v>308.7</v>
+      </c>
+      <c r="F369" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="370" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B370" s="11"/>
+      <c r="B370" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C370" s="5"/>
-      <c r="D370" s="3"/>
-      <c r="E370" s="43"/>
-      <c r="F370" s="7"/>
+      <c r="D370" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E370" s="43">
+        <v>460</v>
+      </c>
+      <c r="F370" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="371" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B371" s="11"/>
+      <c r="B371" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C371" s="5"/>
-      <c r="D371" s="3"/>
-      <c r="E371" s="43"/>
-      <c r="F371" s="7"/>
+      <c r="D371" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E371" s="43">
+        <v>938.9</v>
+      </c>
+      <c r="F371" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="372" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B372" s="11"/>
+      <c r="B372" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C372" s="5"/>
-      <c r="D372" s="3"/>
-      <c r="E372" s="43"/>
-      <c r="F372" s="7"/>
+      <c r="D372" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E372" s="43">
+        <v>638.25</v>
+      </c>
+      <c r="F372" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="373" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B373" s="11"/>
+      <c r="B373" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C373" s="5"/>
-      <c r="D373" s="3"/>
-      <c r="E373" s="43"/>
-      <c r="F373" s="7"/>
+      <c r="D373" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E373" s="43">
+        <v>185</v>
+      </c>
+      <c r="F373" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="374" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B374" s="11"/>
+      <c r="B374" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C374" s="5"/>
-      <c r="D374" s="3"/>
-      <c r="E374" s="43"/>
-      <c r="F374" s="7"/>
+      <c r="D374" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E374" s="43">
+        <v>1863.5</v>
+      </c>
+      <c r="F374" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="375" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B375" s="11"/>
+      <c r="B375" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C375" s="5"/>
-      <c r="D375" s="3"/>
-      <c r="E375" s="43"/>
-      <c r="F375" s="7"/>
+      <c r="D375" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E375" s="43">
+        <v>65</v>
+      </c>
+      <c r="F375" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="376" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B376" s="11"/>
+      <c r="B376" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C376" s="5"/>
-      <c r="D376" s="3"/>
-      <c r="E376" s="43"/>
-      <c r="F376" s="7"/>
+      <c r="D376" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E376" s="43">
+        <v>238.8</v>
+      </c>
+      <c r="F376" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="377" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B377" s="11"/>
+      <c r="B377" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C377" s="5"/>
-      <c r="D377" s="3"/>
-      <c r="E377" s="43"/>
-      <c r="F377" s="7"/>
+      <c r="D377" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E377" s="43">
+        <v>580</v>
+      </c>
+      <c r="F377" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="378" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B378" s="11"/>
+      <c r="B378" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C378" s="5"/>
-      <c r="D378" s="3"/>
-      <c r="E378" s="43"/>
-      <c r="F378" s="7"/>
+      <c r="D378" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E378" s="43">
+        <v>16</v>
+      </c>
+      <c r="F378" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="379" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B379" s="11"/>
+      <c r="B379" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C379" s="5"/>
-      <c r="D379" s="3"/>
-      <c r="E379" s="43"/>
-      <c r="F379" s="7"/>
+      <c r="D379" s="3" t="s">
+        <v>160</v>
+      </c>
+      <c r="E379" s="43">
+        <v>16</v>
+      </c>
+      <c r="F379" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="380" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B380" s="11"/>
+      <c r="B380" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C380" s="5"/>
-      <c r="D380" s="3"/>
-      <c r="E380" s="43"/>
-      <c r="F380" s="7"/>
+      <c r="D380" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E380" s="43">
+        <v>971</v>
+      </c>
+      <c r="F380" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="381" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B381" s="11"/>
+      <c r="B381" s="11" t="s">
+        <v>19</v>
+      </c>
       <c r="C381" s="5"/>
-      <c r="D381" s="3"/>
-      <c r="E381" s="43"/>
-      <c r="F381" s="7"/>
+      <c r="D381" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E381" s="43">
+        <v>28</v>
+      </c>
+      <c r="F381" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="382" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B382" s="11"/>
+      <c r="B382" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C382" s="5"/>
-      <c r="D382" s="3"/>
-      <c r="E382" s="43"/>
-      <c r="F382" s="7"/>
+      <c r="D382" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E382" s="43">
+        <v>140</v>
+      </c>
+      <c r="F382" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="383" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B383" s="11"/>
+      <c r="B383" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="C383" s="5"/>
-      <c r="D383" s="3"/>
-      <c r="E383" s="43"/>
-      <c r="F383" s="7"/>
+      <c r="D383" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E383" s="43">
+        <v>203</v>
+      </c>
+      <c r="F383" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="384" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B384" s="11"/>
+      <c r="B384" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="C384" s="5"/>
-      <c r="D384" s="3"/>
-      <c r="E384" s="43"/>
-      <c r="F384" s="7"/>
+      <c r="D384" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E384" s="43">
+        <v>487</v>
+      </c>
+      <c r="F384" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="385" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B385" s="11"/>
+      <c r="B385" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C385" s="5"/>
-      <c r="D385" s="3"/>
-      <c r="E385" s="43"/>
-      <c r="F385" s="7"/>
+      <c r="D385" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E385" s="43">
+        <v>651.54999999999995</v>
+      </c>
+      <c r="F385" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="386" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B386" s="11"/>
+      <c r="B386" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C386" s="5"/>
-      <c r="D386" s="3"/>
-      <c r="E386" s="43"/>
-      <c r="F386" s="7"/>
+      <c r="D386" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="E386" s="43">
+        <v>100</v>
+      </c>
+      <c r="F386" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="387" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B387" s="11"/>
+      <c r="B387" s="11" t="s">
+        <v>14</v>
+      </c>
       <c r="C387" s="5"/>
-      <c r="D387" s="3"/>
-      <c r="E387" s="43"/>
-      <c r="F387" s="7"/>
+      <c r="D387" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E387" s="43">
+        <v>40</v>
+      </c>
+      <c r="F387" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="388" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B388" s="11"/>
+      <c r="B388" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="C388" s="5"/>
-      <c r="D388" s="3"/>
-      <c r="E388" s="43"/>
-      <c r="F388" s="7"/>
+      <c r="D388" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E388" s="43">
+        <v>643</v>
+      </c>
+      <c r="F388" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="389" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B389" s="11"/>
+      <c r="B389" s="11" t="s">
+        <v>17</v>
+      </c>
       <c r="C389" s="5"/>
-      <c r="D389" s="3"/>
-      <c r="E389" s="43"/>
-      <c r="F389" s="7"/>
+      <c r="D389" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E389" s="43">
+        <v>881</v>
+      </c>
+      <c r="F389" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="390" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B390" s="11"/>
+      <c r="B390" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C390" s="5"/>
-      <c r="D390" s="3"/>
-      <c r="E390" s="43"/>
-      <c r="F390" s="7"/>
+      <c r="D390" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E390" s="43">
+        <v>387</v>
+      </c>
+      <c r="F390" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="391" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B391" s="11"/>
+      <c r="B391" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C391" s="5"/>
-      <c r="D391" s="3"/>
-      <c r="E391" s="43"/>
-      <c r="F391" s="7"/>
+      <c r="D391" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E391" s="43">
+        <v>483.6</v>
+      </c>
+      <c r="F391" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="392" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B392" s="11"/>
+      <c r="B392" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C392" s="5"/>
-      <c r="D392" s="3"/>
-      <c r="E392" s="43"/>
-      <c r="F392" s="7"/>
+      <c r="D392" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E392" s="43">
+        <v>80</v>
+      </c>
+      <c r="F392" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="393" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B393" s="11"/>
+      <c r="B393" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C393" s="5"/>
-      <c r="D393" s="3"/>
-      <c r="E393" s="43"/>
-      <c r="F393" s="7"/>
+      <c r="D393" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E393" s="43">
+        <v>148</v>
+      </c>
+      <c r="F393" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="394" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B394" s="11"/>
+      <c r="B394" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C394" s="5"/>
-      <c r="D394" s="3"/>
-      <c r="E394" s="43"/>
-      <c r="F394" s="7"/>
+      <c r="D394" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E394" s="43">
+        <v>248</v>
+      </c>
+      <c r="F394" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="395" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B395" s="11"/>
+      <c r="B395" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C395" s="5"/>
-      <c r="D395" s="3"/>
-      <c r="E395" s="43"/>
-      <c r="F395" s="7"/>
+      <c r="D395" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E395" s="43">
+        <v>38</v>
+      </c>
+      <c r="F395" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="396" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B396" s="11"/>
+      <c r="B396" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C396" s="5"/>
-      <c r="D396" s="3"/>
-      <c r="E396" s="43"/>
-      <c r="F396" s="7"/>
+      <c r="D396" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E396" s="43">
+        <v>1355</v>
+      </c>
+      <c r="F396" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="397" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B397" s="11"/>
+      <c r="B397" s="11" t="s">
+        <v>7</v>
+      </c>
       <c r="C397" s="5"/>
-      <c r="D397" s="3"/>
-      <c r="E397" s="43"/>
-      <c r="F397" s="7"/>
+      <c r="D397" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="E397" s="43">
+        <v>250</v>
+      </c>
+      <c r="F397" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="398" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B398" s="11"/>
+      <c r="B398" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C398" s="5"/>
-      <c r="D398" s="3"/>
-      <c r="E398" s="43"/>
-      <c r="F398" s="7"/>
+      <c r="D398" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E398" s="43">
+        <v>1393</v>
+      </c>
+      <c r="F398" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="399" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B399" s="11"/>
+      <c r="B399" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C399" s="5"/>
-      <c r="D399" s="3"/>
-      <c r="E399" s="43"/>
-      <c r="F399" s="7"/>
+      <c r="D399" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E399" s="43">
+        <v>4</v>
+      </c>
+      <c r="F399" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="400" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B400" s="11"/>
+      <c r="B400" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C400" s="5"/>
-      <c r="D400" s="3"/>
-      <c r="E400" s="43"/>
-      <c r="F400" s="7"/>
+      <c r="D400" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E400" s="43">
+        <v>690</v>
+      </c>
+      <c r="F400" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="401" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B401" s="11"/>
+      <c r="B401" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C401" s="5"/>
-      <c r="D401" s="3"/>
-      <c r="E401" s="43"/>
-      <c r="F401" s="7"/>
+      <c r="D401" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E401" s="43">
+        <v>1620</v>
+      </c>
+      <c r="F401" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="402" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B402" s="11"/>
+      <c r="B402" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C402" s="5"/>
-      <c r="D402" s="3"/>
-      <c r="E402" s="43"/>
-      <c r="F402" s="7"/>
+      <c r="D402" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E402" s="43">
+        <v>145</v>
+      </c>
+      <c r="F402" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="403" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B403" s="11"/>
+      <c r="B403" s="11" t="s">
+        <v>23</v>
+      </c>
       <c r="C403" s="5"/>
-      <c r="D403" s="3"/>
-      <c r="E403" s="43"/>
-      <c r="F403" s="7"/>
+      <c r="D403" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E403" s="43">
+        <v>120</v>
+      </c>
+      <c r="F403" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="404" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B404" s="11"/>
+      <c r="B404" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C404" s="5"/>
-      <c r="D404" s="3"/>
-      <c r="E404" s="43"/>
-      <c r="F404" s="7"/>
+      <c r="D404" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E404" s="43">
+        <v>100</v>
+      </c>
+      <c r="F404" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="405" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B405" s="11"/>
+      <c r="B405" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C405" s="5"/>
-      <c r="D405" s="3"/>
-      <c r="E405" s="43"/>
-      <c r="F405" s="7"/>
+      <c r="D405" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E405" s="43">
+        <v>195</v>
+      </c>
+      <c r="F405" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="406" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B406" s="11"/>
+      <c r="B406" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C406" s="5"/>
-      <c r="D406" s="3"/>
-      <c r="E406" s="43"/>
-      <c r="F406" s="7"/>
+      <c r="D406" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E406" s="43">
+        <v>200</v>
+      </c>
+      <c r="F406" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="407" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B407" s="11"/>
+      <c r="B407" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C407" s="5"/>
-      <c r="D407" s="3"/>
-      <c r="E407" s="43"/>
-      <c r="F407" s="7"/>
+      <c r="D407" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E407" s="43">
+        <v>220.2</v>
+      </c>
+      <c r="F407" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="408" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B408" s="11"/>
+      <c r="B408" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C408" s="5"/>
-      <c r="D408" s="3"/>
-      <c r="E408" s="43"/>
-      <c r="F408" s="7"/>
+      <c r="D408" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E408" s="43">
+        <v>460</v>
+      </c>
+      <c r="F408" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="409" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B409" s="11"/>
+      <c r="B409" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C409" s="5"/>
-      <c r="D409" s="3"/>
-      <c r="E409" s="43"/>
-      <c r="F409" s="7"/>
+      <c r="D409" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E409" s="43">
+        <v>280</v>
+      </c>
+      <c r="F409" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="410" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B410" s="11"/>
+      <c r="B410" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C410" s="5"/>
-      <c r="D410" s="3"/>
-      <c r="E410" s="43"/>
-      <c r="F410" s="7"/>
+      <c r="D410" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E410" s="43">
+        <v>470</v>
+      </c>
+      <c r="F410" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="411" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B411" s="11"/>
+      <c r="B411" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C411" s="5"/>
-      <c r="D411" s="3"/>
-      <c r="E411" s="43"/>
-      <c r="F411" s="7"/>
+      <c r="D411" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E411" s="43">
+        <v>1770</v>
+      </c>
+      <c r="F411" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="412" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B412" s="11"/>
+      <c r="B412" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C412" s="5"/>
-      <c r="D412" s="3"/>
-      <c r="E412" s="43"/>
-      <c r="F412" s="7"/>
+      <c r="D412" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E412" s="43">
+        <v>220</v>
+      </c>
+      <c r="F412" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="413" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B413" s="11"/>
+      <c r="B413" s="11" t="s">
+        <v>13</v>
+      </c>
       <c r="C413" s="5"/>
-      <c r="D413" s="3"/>
-      <c r="E413" s="43"/>
-      <c r="F413" s="7"/>
+      <c r="D413" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E413" s="43">
+        <v>380</v>
+      </c>
+      <c r="F413" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="414" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B414" s="11"/>
+      <c r="B414" s="11" t="s">
+        <v>8</v>
+      </c>
       <c r="C414" s="5"/>
-      <c r="D414" s="3"/>
-      <c r="E414" s="43"/>
-      <c r="F414" s="7"/>
+      <c r="D414" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E414" s="43">
+        <v>150</v>
+      </c>
+      <c r="F414" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="415" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B415" s="11"/>
+      <c r="B415" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C415" s="5"/>
-      <c r="D415" s="3"/>
-      <c r="E415" s="43"/>
-      <c r="F415" s="7"/>
+      <c r="D415" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E415" s="43">
+        <v>189</v>
+      </c>
+      <c r="F415" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="416" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B416" s="11"/>
+      <c r="B416" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C416" s="5"/>
-      <c r="D416" s="3"/>
-      <c r="E416" s="43"/>
-      <c r="F416" s="7"/>
+      <c r="D416" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E416" s="43">
+        <v>75</v>
+      </c>
+      <c r="F416" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="417" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B417" s="11"/>
+      <c r="B417" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C417" s="5"/>
-      <c r="D417" s="3"/>
-      <c r="E417" s="43"/>
-      <c r="F417" s="7"/>
+      <c r="D417" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E417" s="43">
+        <v>50</v>
+      </c>
+      <c r="F417" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="418" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B418" s="11"/>
+      <c r="B418" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C418" s="5"/>
-      <c r="D418" s="3"/>
-      <c r="E418" s="43"/>
-      <c r="F418" s="7"/>
+      <c r="D418" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E418" s="43">
+        <v>154</v>
+      </c>
+      <c r="F418" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="419" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B419" s="11"/>
+      <c r="B419" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C419" s="5"/>
-      <c r="D419" s="3"/>
-      <c r="E419" s="43"/>
-      <c r="F419" s="7"/>
+      <c r="D419" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E419" s="43">
+        <v>1066</v>
+      </c>
+      <c r="F419" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="420" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B420" s="11"/>
+      <c r="B420" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C420" s="5"/>
-      <c r="D420" s="3"/>
-      <c r="E420" s="43"/>
-      <c r="F420" s="7"/>
+      <c r="D420" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E420" s="43">
+        <v>500</v>
+      </c>
+      <c r="F420" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="421" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B421" s="11"/>
+      <c r="B421" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C421" s="5"/>
-      <c r="D421" s="3"/>
-      <c r="E421" s="43"/>
-      <c r="F421" s="7"/>
+      <c r="D421" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E421" s="43">
+        <v>120</v>
+      </c>
+      <c r="F421" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="422" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B422" s="11"/>
+      <c r="B422" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C422" s="5"/>
-      <c r="D422" s="3"/>
-      <c r="E422" s="43"/>
-      <c r="F422" s="7"/>
+      <c r="D422" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E422" s="43">
+        <v>240</v>
+      </c>
+      <c r="F422" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="423" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B423" s="11"/>
+      <c r="B423" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C423" s="5"/>
-      <c r="D423" s="3"/>
-      <c r="E423" s="43"/>
-      <c r="F423" s="7"/>
+      <c r="D423" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E423" s="43">
+        <v>80</v>
+      </c>
+      <c r="F423" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="424" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B424" s="11"/>
+      <c r="B424" s="11" t="s">
+        <v>10</v>
+      </c>
       <c r="C424" s="5"/>
-      <c r="D424" s="3"/>
-      <c r="E424" s="43"/>
-      <c r="F424" s="7"/>
+      <c r="D424" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="E424" s="43">
+        <v>70</v>
+      </c>
+      <c r="F424" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="425" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B425" s="11"/>
+      <c r="B425" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C425" s="5"/>
-      <c r="D425" s="3"/>
-      <c r="E425" s="43"/>
-      <c r="F425" s="7"/>
+      <c r="D425" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E425" s="43">
+        <v>73</v>
+      </c>
+      <c r="F425" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="426" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B426" s="11"/>
+      <c r="B426" s="11" t="s">
+        <v>4</v>
+      </c>
       <c r="C426" s="5"/>
-      <c r="D426" s="3"/>
-      <c r="E426" s="43"/>
-      <c r="F426" s="7"/>
+      <c r="D426" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E426" s="43">
+        <v>200</v>
+      </c>
+      <c r="F426" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="427" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B427" s="11"/>
+      <c r="B427" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C427" s="5"/>
-      <c r="D427" s="3"/>
-      <c r="E427" s="43"/>
-      <c r="F427" s="7"/>
+      <c r="D427" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E427" s="43">
+        <v>510</v>
+      </c>
+      <c r="F427" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="428" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B428" s="11"/>
+      <c r="B428" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C428" s="5"/>
-      <c r="D428" s="3"/>
-      <c r="E428" s="43"/>
-      <c r="F428" s="7"/>
+      <c r="D428" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E428" s="43">
+        <v>6243.77</v>
+      </c>
+      <c r="F428" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="429" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B429" s="11"/>
+      <c r="B429" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C429" s="5"/>
-      <c r="D429" s="3"/>
-      <c r="E429" s="43"/>
-      <c r="F429" s="7"/>
+      <c r="D429" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E429" s="43">
+        <v>2131.3000000000002</v>
+      </c>
+      <c r="F429" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="430" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B430" s="11"/>
+      <c r="B430" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C430" s="5"/>
-      <c r="D430" s="3"/>
-      <c r="E430" s="43"/>
-      <c r="F430" s="7"/>
+      <c r="D430" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="E430" s="43">
+        <v>1510</v>
+      </c>
+      <c r="F430" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="431" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B431" s="11"/>
+      <c r="B431" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C431" s="5"/>
-      <c r="D431" s="3"/>
-      <c r="E431" s="43"/>
-      <c r="F431" s="7"/>
+      <c r="D431" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E431" s="43">
+        <v>80</v>
+      </c>
+      <c r="F431" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="432" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B432" s="11"/>
+      <c r="B432" s="11" t="s">
+        <v>34</v>
+      </c>
       <c r="C432" s="5"/>
-      <c r="D432" s="3"/>
-      <c r="E432" s="43"/>
-      <c r="F432" s="7"/>
+      <c r="D432" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E432" s="43">
+        <v>144</v>
+      </c>
+      <c r="F432" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="433" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B433" s="11"/>
+      <c r="B433" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C433" s="5"/>
-      <c r="D433" s="3"/>
-      <c r="E433" s="43"/>
-      <c r="F433" s="7"/>
+      <c r="D433" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E433" s="43">
+        <v>200</v>
+      </c>
+      <c r="F433" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="434" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B434" s="11"/>
+      <c r="B434" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C434" s="5"/>
-      <c r="D434" s="3"/>
-      <c r="E434" s="43"/>
-      <c r="F434" s="7"/>
+      <c r="D434" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E434" s="43">
+        <v>800</v>
+      </c>
+      <c r="F434" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="435" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B435" s="11"/>
+      <c r="B435" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C435" s="5"/>
-      <c r="D435" s="3"/>
-      <c r="E435" s="43"/>
-      <c r="F435" s="7"/>
+      <c r="D435" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E435" s="43">
+        <v>50</v>
+      </c>
+      <c r="F435" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="436" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B436" s="11"/>
+      <c r="B436" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C436" s="5"/>
-      <c r="D436" s="3"/>
-      <c r="E436" s="43"/>
-      <c r="F436" s="7"/>
+      <c r="D436" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E436" s="43">
+        <v>3500</v>
+      </c>
+      <c r="F436" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="437" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B437" s="11"/>
+      <c r="B437" s="11" t="s">
+        <v>82</v>
+      </c>
       <c r="C437" s="5"/>
-      <c r="D437" s="3"/>
-      <c r="E437" s="43"/>
-      <c r="F437" s="7"/>
+      <c r="D437" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E437" s="43">
+        <v>3250</v>
+      </c>
+      <c r="F437" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="438" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B438" s="11"/>
+      <c r="B438" s="11" t="s">
+        <v>25</v>
+      </c>
       <c r="C438" s="5"/>
-      <c r="D438" s="3"/>
-      <c r="E438" s="43"/>
-      <c r="F438" s="7"/>
+      <c r="D438" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E438" s="43">
+        <v>35</v>
+      </c>
+      <c r="F438" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="439" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B439" s="11"/>
+      <c r="B439" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C439" s="5"/>
-      <c r="D439" s="3"/>
-      <c r="E439" s="43"/>
-      <c r="F439" s="7"/>
+      <c r="D439" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E439" s="43">
+        <v>175</v>
+      </c>
+      <c r="F439" s="7">
+        <v>46082</v>
+      </c>
     </row>
     <row r="440" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B440" s="11"/>
+      <c r="B440" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C440" s="5"/>
-      <c r="D440" s="3"/>
-      <c r="E440" s="43"/>
-      <c r="F440" s="7"/>
+      <c r="D440" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E440" s="43">
+        <v>847</v>
+      </c>
+      <c r="F440" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="441" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B441" s="11"/>
+      <c r="B441" s="11" t="s">
+        <v>21</v>
+      </c>
       <c r="C441" s="5"/>
-      <c r="D441" s="3"/>
-      <c r="E441" s="43"/>
-      <c r="F441" s="7"/>
+      <c r="D441" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E441" s="43">
+        <v>302</v>
+      </c>
+      <c r="F441" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="442" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B442" s="11"/>
+      <c r="B442" s="11" t="s">
+        <v>11</v>
+      </c>
       <c r="C442" s="5"/>
-      <c r="D442" s="3"/>
-      <c r="E442" s="43"/>
-      <c r="F442" s="7"/>
+      <c r="D442" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E442" s="43">
+        <v>730</v>
+      </c>
+      <c r="F442" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="443" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B443" s="11"/>
+      <c r="B443" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C443" s="5"/>
-      <c r="D443" s="3"/>
-      <c r="E443" s="43"/>
-      <c r="F443" s="7"/>
+      <c r="D443" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E443" s="43">
+        <v>215</v>
+      </c>
+      <c r="F443" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="444" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B444" s="11"/>
+      <c r="B444" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C444" s="5"/>
-      <c r="D444" s="3"/>
-      <c r="E444" s="43"/>
-      <c r="F444" s="7"/>
+      <c r="D444" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E444" s="43">
+        <v>170</v>
+      </c>
+      <c r="F444" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="445" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B445" s="11"/>
+      <c r="B445" s="11" t="s">
+        <v>22</v>
+      </c>
       <c r="C445" s="5"/>
-      <c r="D445" s="3"/>
-      <c r="E445" s="43"/>
-      <c r="F445" s="7"/>
+      <c r="D445" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E445" s="43">
+        <v>50</v>
+      </c>
+      <c r="F445" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="446" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B446" s="11"/>
+      <c r="B446" s="11" t="s">
+        <v>117</v>
+      </c>
       <c r="C446" s="5"/>
-      <c r="D446" s="3"/>
-      <c r="E446" s="43"/>
-      <c r="F446" s="7"/>
+      <c r="D446" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E446" s="43">
+        <v>55</v>
+      </c>
+      <c r="F446" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="447" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B447" s="11"/>
+      <c r="B447" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C447" s="5"/>
-      <c r="D447" s="3"/>
-      <c r="E447" s="43"/>
-      <c r="F447" s="7"/>
+      <c r="D447" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E447" s="43">
+        <v>1141</v>
+      </c>
+      <c r="F447" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="448" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B448" s="11"/>
+      <c r="B448" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C448" s="5"/>
-      <c r="D448" s="3"/>
-      <c r="E448" s="43"/>
-      <c r="F448" s="7"/>
+      <c r="D448" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E448" s="43">
+        <v>500</v>
+      </c>
+      <c r="F448" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="449" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B449" s="11"/>
+      <c r="B449" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C449" s="5"/>
-      <c r="D449" s="3"/>
-      <c r="E449" s="43"/>
-      <c r="F449" s="7"/>
+      <c r="D449" s="3" t="s">
+        <v>158</v>
+      </c>
+      <c r="E449" s="43">
+        <v>300</v>
+      </c>
+      <c r="F449" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="450" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B450" s="11"/>
+      <c r="B450" s="11" t="s">
+        <v>29</v>
+      </c>
       <c r="C450" s="5"/>
-      <c r="D450" s="3"/>
-      <c r="E450" s="43"/>
-      <c r="F450" s="7"/>
+      <c r="D450" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E450" s="43">
+        <v>40</v>
+      </c>
+      <c r="F450" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="451" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B451" s="11"/>
+      <c r="B451" s="11" t="s">
+        <v>15</v>
+      </c>
       <c r="C451" s="5"/>
-      <c r="D451" s="3"/>
-      <c r="E451" s="43"/>
-      <c r="F451" s="7"/>
+      <c r="D451" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="E451" s="43">
+        <v>200</v>
+      </c>
+      <c r="F451" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="452" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B452" s="11"/>
+      <c r="B452" s="11" t="s">
+        <v>5</v>
+      </c>
       <c r="C452" s="5"/>
-      <c r="D452" s="3"/>
-      <c r="E452" s="43"/>
-      <c r="F452" s="7"/>
+      <c r="D452" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E452" s="43">
+        <v>100</v>
+      </c>
+      <c r="F452" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="453" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B453" s="11"/>
+      <c r="B453" s="11" t="s">
+        <v>24</v>
+      </c>
       <c r="C453" s="5"/>
-      <c r="D453" s="3"/>
-      <c r="E453" s="43"/>
-      <c r="F453" s="7"/>
+      <c r="D453" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E453" s="43">
+        <v>1449</v>
+      </c>
+      <c r="F453" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="454" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B454" s="11"/>
+      <c r="B454" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C454" s="5"/>
-      <c r="D454" s="3"/>
-      <c r="E454" s="43"/>
-      <c r="F454" s="7"/>
+      <c r="D454" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E454" s="43">
+        <v>750</v>
+      </c>
+      <c r="F454" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="455" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B455" s="11"/>
+      <c r="B455" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C455" s="5"/>
-      <c r="D455" s="3"/>
-      <c r="E455" s="43"/>
-      <c r="F455" s="7"/>
+      <c r="D455" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E455" s="43">
+        <v>1130</v>
+      </c>
+      <c r="F455" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="456" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B456" s="11"/>
+      <c r="B456" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C456" s="5"/>
-      <c r="D456" s="3"/>
-      <c r="E456" s="43"/>
-      <c r="F456" s="7"/>
+      <c r="D456" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E456" s="43">
+        <v>650</v>
+      </c>
+      <c r="F456" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="457" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B457" s="11"/>
+      <c r="B457" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C457" s="5"/>
-      <c r="D457" s="3"/>
-      <c r="E457" s="43"/>
-      <c r="F457" s="7"/>
+      <c r="D457" s="3" t="s">
+        <v>118</v>
+      </c>
+      <c r="E457" s="43">
+        <v>350</v>
+      </c>
+      <c r="F457" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="458" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B458" s="11"/>
+      <c r="B458" s="11" t="s">
+        <v>3</v>
+      </c>
       <c r="C458" s="5"/>
-      <c r="D458" s="3"/>
-      <c r="E458" s="43"/>
-      <c r="F458" s="7"/>
+      <c r="D458" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E458" s="43">
+        <v>3912</v>
+      </c>
+      <c r="F458" s="7">
+        <v>46143</v>
+      </c>
     </row>
     <row r="459" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B459" s="11"/>

</xml_diff>

<commit_message>
Atualizacao automatica 2026-05-07 11:00
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1109" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3B71718C-E7FA-4FF4-8117-07FD318F6E2C}"/>
+  <xr:revisionPtr revIDLastSave="1115" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A6139DC-8521-4607-961A-5B98739BE878}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3078" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3078" uniqueCount="183">
   <si>
     <t>Custo</t>
   </si>
@@ -487,9 +487,6 @@
     <t>NOVA FREIOS E PEÇAS</t>
   </si>
   <si>
-    <t>PNEUS MAX</t>
-  </si>
-  <si>
     <t>LONAS VINIFORTE</t>
   </si>
   <si>
@@ -506,9 +503,6 @@
   </si>
   <si>
     <t>SILVA CARROCERIA</t>
-  </si>
-  <si>
-    <t>PNEU MAX</t>
   </si>
   <si>
     <t>BORRACHARIA NITEROI</t>
@@ -41132,7 +41126,7 @@
       </c>
       <c r="C99" s="5"/>
       <c r="D99" s="3" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="E99" s="43">
         <v>505</v>
@@ -41192,7 +41186,7 @@
       </c>
       <c r="C103" s="5"/>
       <c r="D103" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E103" s="43">
         <v>170</v>
@@ -41207,7 +41201,7 @@
       </c>
       <c r="C104" s="5"/>
       <c r="D104" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="E104" s="43">
         <v>416</v>
@@ -41222,7 +41216,7 @@
       </c>
       <c r="C105" s="5"/>
       <c r="D105" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E105" s="43">
         <v>1100</v>
@@ -41248,11 +41242,11 @@
     </row>
     <row r="107" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B107" s="11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C107" s="5"/>
       <c r="D107" s="25" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="E107" s="20">
         <v>1590</v>
@@ -41297,7 +41291,7 @@
       </c>
       <c r="C110" s="5"/>
       <c r="D110" s="3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E110" s="43">
         <v>2735.31</v>
@@ -41657,7 +41651,7 @@
       </c>
       <c r="C134" s="5"/>
       <c r="D134" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E134" s="43">
         <v>310</v>
@@ -41672,7 +41666,7 @@
       </c>
       <c r="C135" s="5"/>
       <c r="D135" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E135" s="43">
         <v>1350</v>
@@ -41687,7 +41681,7 @@
       </c>
       <c r="C136" s="5"/>
       <c r="D136" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E136" s="43">
         <v>190</v>
@@ -41702,7 +41696,7 @@
       </c>
       <c r="C137" s="5"/>
       <c r="D137" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E137" s="43">
         <v>720</v>
@@ -41717,7 +41711,7 @@
       </c>
       <c r="C138" s="5"/>
       <c r="D138" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E138" s="43">
         <v>160</v>
@@ -41732,7 +41726,7 @@
       </c>
       <c r="C139" s="5"/>
       <c r="D139" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E139" s="43">
         <v>180</v>
@@ -41747,7 +41741,7 @@
       </c>
       <c r="C140" s="5"/>
       <c r="D140" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E140" s="43">
         <v>2710</v>
@@ -42032,7 +42026,7 @@
       </c>
       <c r="C159" s="5"/>
       <c r="D159" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E159" s="43">
         <v>1508</v>
@@ -42062,7 +42056,7 @@
       </c>
       <c r="C161" s="5"/>
       <c r="D161" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E161" s="43">
         <v>30</v>
@@ -42077,7 +42071,7 @@
       </c>
       <c r="C162" s="5"/>
       <c r="D162" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E162" s="43">
         <v>3635</v>
@@ -42092,7 +42086,7 @@
       </c>
       <c r="C163" s="5"/>
       <c r="D163" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E163" s="43">
         <v>4200</v>
@@ -42107,7 +42101,7 @@
       </c>
       <c r="C164" s="5"/>
       <c r="D164" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E164" s="43">
         <v>1497</v>
@@ -42122,7 +42116,7 @@
       </c>
       <c r="C165" s="5"/>
       <c r="D165" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E165" s="43">
         <v>2944</v>
@@ -42223,7 +42217,7 @@
     </row>
     <row r="172" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B172" s="11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C172" s="5"/>
       <c r="D172" s="3" t="s">
@@ -42287,7 +42281,7 @@
       </c>
       <c r="C176" s="5"/>
       <c r="D176" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E176" s="43">
         <v>1200</v>
@@ -42302,7 +42296,7 @@
       </c>
       <c r="C177" s="5"/>
       <c r="D177" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E177" s="43">
         <v>280</v>
@@ -42422,7 +42416,7 @@
       </c>
       <c r="C185" s="5"/>
       <c r="D185" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E185" s="43">
         <v>224.18</v>
@@ -42452,7 +42446,7 @@
       </c>
       <c r="C187" s="5"/>
       <c r="D187" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E187" s="43">
         <v>250</v>
@@ -42557,7 +42551,7 @@
       </c>
       <c r="C194" s="5"/>
       <c r="D194" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E194" s="43">
         <v>80</v>
@@ -42617,7 +42611,7 @@
       </c>
       <c r="C198" s="5"/>
       <c r="D198" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E198" s="43">
         <v>200</v>
@@ -42632,7 +42626,7 @@
       </c>
       <c r="C199" s="5"/>
       <c r="D199" s="3" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E199" s="43">
         <v>150</v>
@@ -42748,7 +42742,7 @@
     </row>
     <row r="207" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B207" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C207" s="5"/>
       <c r="D207" s="3" t="s">
@@ -42827,7 +42821,7 @@
       </c>
       <c r="C212" s="5"/>
       <c r="D212" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E212" s="43">
         <v>100</v>
@@ -42868,7 +42862,7 @@
     </row>
     <row r="215" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B215" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C215" s="5"/>
       <c r="D215" s="3" t="s">
@@ -42887,7 +42881,7 @@
       </c>
       <c r="C216" s="5"/>
       <c r="D216" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E216" s="43">
         <v>420</v>
@@ -42928,11 +42922,11 @@
     </row>
     <row r="219" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B219" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C219" s="5"/>
       <c r="D219" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E219" s="43">
         <v>30</v>
@@ -43018,7 +43012,7 @@
     </row>
     <row r="225" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B225" s="11" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C225" s="5"/>
       <c r="D225" s="3" t="s">
@@ -43183,7 +43177,7 @@
     </row>
     <row r="236" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B236" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C236" s="5"/>
       <c r="D236" s="3" t="s">
@@ -43307,7 +43301,7 @@
       </c>
       <c r="C244" s="5"/>
       <c r="D244" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E244" s="43">
         <v>78</v>
@@ -43412,7 +43406,7 @@
       </c>
       <c r="C251" s="5"/>
       <c r="D251" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E251" s="43">
         <v>580</v>
@@ -43457,7 +43451,7 @@
       </c>
       <c r="C254" s="5"/>
       <c r="D254" s="3" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="E254" s="43">
         <v>12156</v>
@@ -43472,7 +43466,7 @@
       </c>
       <c r="C255" s="5"/>
       <c r="D255" s="3" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="E255" s="43">
         <v>16800</v>
@@ -43483,11 +43477,11 @@
     </row>
     <row r="256" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B256" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C256" s="5"/>
       <c r="D256" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E256" s="43">
         <v>97</v>
@@ -43738,7 +43732,7 @@
     </row>
     <row r="273" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B273" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C273" s="5"/>
       <c r="D273" s="3" t="s">
@@ -43905,7 +43899,7 @@
       </c>
       <c r="C284" s="5"/>
       <c r="D284" s="3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="E284" s="43">
         <v>7000</v>
@@ -43965,7 +43959,7 @@
       </c>
       <c r="C288" s="5"/>
       <c r="D288" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E288" s="43">
         <v>432</v>
@@ -44130,7 +44124,7 @@
       </c>
       <c r="C299" s="5"/>
       <c r="D299" s="3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="E299" s="43">
         <v>50</v>
@@ -44145,7 +44139,7 @@
       </c>
       <c r="C300" s="5"/>
       <c r="D300" s="3" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="E300" s="43">
         <v>65</v>
@@ -44325,7 +44319,7 @@
       </c>
       <c r="C312" s="5"/>
       <c r="D312" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E312" s="43">
         <v>1460</v>
@@ -44385,7 +44379,7 @@
       </c>
       <c r="C316" s="5"/>
       <c r="D316" s="3" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="E316" s="43">
         <v>2096</v>
@@ -44475,7 +44469,7 @@
       </c>
       <c r="C322" s="5"/>
       <c r="D322" s="3" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="E322" s="43">
         <v>213.6</v>
@@ -44625,7 +44619,7 @@
       </c>
       <c r="C332" s="5"/>
       <c r="D332" s="3" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="E332" s="43">
         <v>200</v>
@@ -44640,7 +44634,7 @@
       </c>
       <c r="C333" s="5"/>
       <c r="D333" s="3" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="E333" s="43">
         <v>161.30000000000001</v>
@@ -44655,7 +44649,7 @@
       </c>
       <c r="C334" s="5"/>
       <c r="D334" s="3" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E334" s="43">
         <v>110</v>
@@ -44685,7 +44679,7 @@
       </c>
       <c r="C336" s="5"/>
       <c r="D336" s="3" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E336" s="43">
         <v>80</v>
@@ -44700,7 +44694,7 @@
       </c>
       <c r="C337" s="5"/>
       <c r="D337" s="3" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E337" s="43">
         <v>30</v>
@@ -44730,7 +44724,7 @@
       </c>
       <c r="C339" s="5"/>
       <c r="D339" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E339" s="43">
         <v>2967</v>
@@ -44790,7 +44784,7 @@
       </c>
       <c r="C343" s="5"/>
       <c r="D343" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E343" s="43">
         <v>510</v>
@@ -44835,7 +44829,7 @@
       </c>
       <c r="C346" s="5"/>
       <c r="D346" s="3" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="E346" s="43">
         <v>10002</v>
@@ -44846,7 +44840,7 @@
     </row>
     <row r="347" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B347" s="11" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C347" s="5"/>
       <c r="D347" s="3"/>
@@ -44863,7 +44857,7 @@
       </c>
       <c r="C348" s="5"/>
       <c r="D348" s="3" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E348" s="43">
         <v>95</v>
@@ -44979,11 +44973,11 @@
     </row>
     <row r="356" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B356" s="11" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C356" s="5"/>
       <c r="D356" s="3" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E356" s="43">
         <v>30</v>
@@ -45058,7 +45052,7 @@
       </c>
       <c r="C361" s="5"/>
       <c r="D361" s="3" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="E361" s="43">
         <v>2858</v>
@@ -45073,7 +45067,7 @@
       </c>
       <c r="C362" s="5"/>
       <c r="D362" s="3" t="s">
-        <v>148</v>
+        <v>83</v>
       </c>
       <c r="E362" s="43">
         <v>2150</v>
@@ -45313,7 +45307,7 @@
       </c>
       <c r="C378" s="5"/>
       <c r="D378" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E378" s="43">
         <v>16</v>
@@ -45328,7 +45322,7 @@
       </c>
       <c r="C379" s="5"/>
       <c r="D379" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E379" s="43">
         <v>16</v>
@@ -45598,7 +45592,7 @@
       </c>
       <c r="C397" s="5"/>
       <c r="D397" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E397" s="43">
         <v>250</v>
@@ -45643,7 +45637,7 @@
       </c>
       <c r="C400" s="5"/>
       <c r="D400" s="3" t="s">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E400" s="43">
         <v>690</v>
@@ -45688,7 +45682,7 @@
       </c>
       <c r="C403" s="5"/>
       <c r="D403" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E403" s="43">
         <v>120</v>
@@ -45838,7 +45832,7 @@
       </c>
       <c r="C413" s="5"/>
       <c r="D413" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E413" s="43">
         <v>380</v>
@@ -46093,7 +46087,7 @@
       </c>
       <c r="C430" s="5"/>
       <c r="D430" s="3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E430" s="43">
         <v>1510</v>
@@ -46378,7 +46372,7 @@
       </c>
       <c r="C449" s="5"/>
       <c r="D449" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E449" s="43">
         <v>300</v>
@@ -63923,7 +63917,7 @@
       </c>
       <c r="C2945" s="24"/>
       <c r="D2945" s="24" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E2945" s="46">
         <v>40</v>

</xml_diff>

<commit_message>
Atualiza dashboard para Streamlit
</commit_message>
<xml_diff>
--- a/data/manutencao.xlsx
+++ b/data/manutencao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jrferragens-my.sharepoint.com/personal/gabriela_costa_jrferragens_com/Documents/Transportes/ARQUIVOS TRANSPORTE/DASHBOARD/DASHBOARD/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1115" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A6139DC-8521-4607-961A-5B98739BE878}"/>
+  <xr:revisionPtr revIDLastSave="1189" documentId="13_ncr:1_{1AC0764F-B6E5-4591-8DB7-B0B61D6064FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DDD0C52D-5343-4197-8915-DAFF467E1586}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="2025" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
+    <workbookView xWindow="28680" yWindow="1050" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{E3C74772-B78D-41DC-AF47-91104267B3E5}"/>
   </bookViews>
   <sheets>
     <sheet name="2025" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3078" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3111" uniqueCount="186">
   <si>
     <t>Custo</t>
   </si>
@@ -590,6 +590,15 @@
   </si>
   <si>
     <t>bombas injetoras</t>
+  </si>
+  <si>
+    <t>HJ PNEUS</t>
+  </si>
+  <si>
+    <t>BORRACHARIA</t>
+  </si>
+  <si>
+    <t>BORRACHARIA BANDEIRANTES</t>
   </si>
 </sst>
 </file>
@@ -17468,10 +17477,19 @@
       </c>
     </row>
     <row r="1080" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B1080" s="25" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1080" s="7"/>
+      <c r="B1080" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C1080" s="5"/>
+      <c r="D1080" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E1080" s="43">
+        <v>54</v>
+      </c>
+      <c r="F1080" s="7">
+        <v>45992</v>
+      </c>
     </row>
     <row r="1081" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1081" s="11"/>
@@ -46517,116 +46535,243 @@
       </c>
     </row>
     <row r="459" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B459" s="11"/>
+      <c r="B459" s="25" t="s">
+        <v>27</v>
+      </c>
       <c r="C459" s="5"/>
-      <c r="D459" s="3"/>
-      <c r="E459" s="43"/>
-      <c r="F459" s="7"/>
+      <c r="D459" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E459" s="43">
+        <v>160</v>
+      </c>
+      <c r="F459" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="460" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B460" s="11"/>
+      <c r="B460" s="11" t="s">
+        <v>28</v>
+      </c>
       <c r="C460" s="5"/>
-      <c r="D460" s="3"/>
-      <c r="E460" s="43"/>
-      <c r="F460" s="7"/>
+      <c r="D460" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E460" s="43">
+        <v>755</v>
+      </c>
+      <c r="F460" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="461" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B461" s="11"/>
+      <c r="B461" s="11" t="s">
+        <v>18</v>
+      </c>
       <c r="C461" s="5"/>
-      <c r="D461" s="3"/>
-      <c r="E461" s="43"/>
-      <c r="F461" s="7"/>
+      <c r="D461" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E461" s="43">
+        <v>250</v>
+      </c>
+      <c r="F461" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="462" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B462" s="11"/>
+      <c r="B462" s="11" t="s">
+        <v>27</v>
+      </c>
       <c r="C462" s="5"/>
-      <c r="D462" s="3"/>
-      <c r="E462" s="43"/>
-      <c r="F462" s="7"/>
+      <c r="D462" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E462" s="43">
+        <v>160</v>
+      </c>
+      <c r="F462" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="463" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B463" s="11"/>
+      <c r="B463" s="11" t="s">
+        <v>6</v>
+      </c>
       <c r="C463" s="5"/>
-      <c r="D463" s="3"/>
-      <c r="E463" s="43"/>
-      <c r="F463" s="7"/>
+      <c r="D463" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="E463" s="43">
+        <v>70</v>
+      </c>
+      <c r="F463" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="464" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B464" s="11"/>
+      <c r="B464" s="11" t="s">
+        <v>31</v>
+      </c>
       <c r="C464" s="5"/>
-      <c r="D464" s="3"/>
-      <c r="E464" s="43"/>
-      <c r="F464" s="7"/>
+      <c r="D464" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="E464" s="43">
+        <v>33</v>
+      </c>
+      <c r="F464" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="465" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B465" s="11"/>
+      <c r="B465" s="11" t="s">
+        <v>26</v>
+      </c>
       <c r="C465" s="5"/>
-      <c r="D465" s="3"/>
-      <c r="E465" s="43"/>
-      <c r="F465" s="7"/>
+      <c r="D465" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E465" s="43">
+        <v>910</v>
+      </c>
+      <c r="F465" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="466" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B466" s="11"/>
+      <c r="B466" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C466" s="5"/>
-      <c r="D466" s="3"/>
-      <c r="E466" s="43"/>
-      <c r="F466" s="7"/>
+      <c r="D466" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E466" s="43">
+        <v>1370</v>
+      </c>
+      <c r="F466" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="467" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B467" s="11"/>
+      <c r="B467" s="11" t="s">
+        <v>146</v>
+      </c>
       <c r="C467" s="5"/>
-      <c r="D467" s="3"/>
-      <c r="E467" s="43"/>
-      <c r="F467" s="7"/>
+      <c r="D467" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E467" s="43">
+        <v>720</v>
+      </c>
+      <c r="F467" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="468" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B468" s="11"/>
+      <c r="B468" s="11" t="s">
+        <v>30</v>
+      </c>
       <c r="C468" s="5"/>
-      <c r="D468" s="3"/>
-      <c r="E468" s="43"/>
-      <c r="F468" s="7"/>
+      <c r="D468" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E468" s="43">
+        <v>1500</v>
+      </c>
+      <c r="F468" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="469" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B469" s="11"/>
+      <c r="B469" s="11" t="s">
+        <v>20</v>
+      </c>
       <c r="C469" s="5"/>
-      <c r="D469" s="3"/>
-      <c r="E469" s="43"/>
-      <c r="F469" s="7"/>
+      <c r="D469" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E469" s="43">
+        <v>460</v>
+      </c>
+      <c r="F469" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="470" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B470" s="11"/>
+      <c r="B470" s="11" t="s">
+        <v>180</v>
+      </c>
       <c r="C470" s="5"/>
-      <c r="D470" s="3"/>
-      <c r="E470" s="43"/>
-      <c r="F470" s="7"/>
+      <c r="D470" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="E470" s="43">
+        <v>50</v>
+      </c>
+      <c r="F470" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="471" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B471" s="11"/>
+      <c r="B471" s="11" t="s">
+        <v>180</v>
+      </c>
       <c r="C471" s="5"/>
-      <c r="D471" s="3"/>
-      <c r="E471" s="43"/>
-      <c r="F471" s="7"/>
+      <c r="D471" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="E471" s="43">
+        <v>30</v>
+      </c>
+      <c r="F471" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="472" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B472" s="11"/>
-      <c r="C472" s="5"/>
-      <c r="D472" s="3"/>
-      <c r="E472" s="43"/>
-      <c r="F472" s="7"/>
+      <c r="B472" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D472" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="E472" s="44">
+        <v>161.30000000000001</v>
+      </c>
+      <c r="F472" s="39">
+        <v>46082</v>
+      </c>
     </row>
     <row r="473" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B473" s="11"/>
+      <c r="B473" s="11" t="s">
+        <v>9</v>
+      </c>
       <c r="C473" s="5"/>
-      <c r="D473" s="3"/>
-      <c r="E473" s="43"/>
-      <c r="F473" s="7"/>
+      <c r="D473" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="E473" s="43">
+        <v>46</v>
+      </c>
+      <c r="F473" s="7">
+        <v>46054</v>
+      </c>
     </row>
     <row r="474" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B474" s="11"/>
+      <c r="B474" s="11" t="s">
+        <v>34</v>
+      </c>
       <c r="C474" s="5"/>
-      <c r="D474" s="3"/>
-      <c r="E474" s="43"/>
-      <c r="F474" s="7"/>
+      <c r="D474" s="25" t="s">
+        <v>94</v>
+      </c>
+      <c r="E474" s="43">
+        <v>144</v>
+      </c>
+      <c r="F474" s="7">
+        <v>46113</v>
+      </c>
     </row>
     <row r="475" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B475" s="11"/>

</xml_diff>